<commit_message>
feat(news): publish 2026-10-26 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-25-en.xlsx
+++ b/docs/exports/week-2026-10-25-en.xlsx
@@ -166,58 +166,60 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Typhoon grid restoration and smart-factory systems
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">By October 24 afternoon, Taipower reported more than 340,000 accounts affected and over 90% restored, including salt-related insulation problems in Yunlin. Chunghwa Telecom separately formed an intelligent-vision subsidiary, with no related fab downtime or new device installation figures.</t>
+            <t xml:space="preserve">Storm recovery, factory power and smart systems
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taipower reported more than 340,000 accounts affected nationwide on October 24, and Yilan declared restoration to over 30,000 affected household accounts by 4 p.m. October 25. The dates and geographies differ, with no fab downtime data. Chunghwa Telecom separately formed an intelligent-vision subsidiary without industrial installation figures.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="130" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Southeast Asian cable tender and Malaysia data-center intentions
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">The MViSTA developer estimates a roughly US$400 million cable with service targeted for late 2028. Malaysia's prime minister separately cited a US$50 billion AI/data-center investment intention on October 24, with media naming SoftBank's Masayoshi Son on October 25. Neither plan supplies approved construction or energization milestones; neither is realized spending.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">Oct 22, Oct 24</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="98" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">03</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Southeast Asian subsea cable and Vietnam campus planning
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">The developer of the proposed 2,500-km MViSTA cable connecting four Southeast Asian countries reported ongoing bidding, an estimated US$400 million cost and a late-2028 target. A USTDA-backed data-center feasibility study in Ho Chi Minh City is a separate undertaking.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C5" s="6">
-        <v>46317</v>
-      </c>
-    </row>
-    <row r="6" ht="98" customHeight="1">
+    <row r="6" ht="114" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">04</t>
@@ -232,21 +234,23 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">GSEO-3M optical interconnect and earnings update
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">GSEO reported about NT$434 million in self-compiled September parent-attributable profit, down 15%, while reporting said the roughly NT$4.813 billion 3M placement proceeds arrived. EBO and CPO product qualification remains pending.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C6" s="6">
-        <v>46318</v>
+            <t xml:space="preserve">Taiwan optical interconnect and high-tech equipment logistics
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">GSEO and 3M's interconnect collaboration has not published qualified production deliveries. On October 25 EVA Air cited sustained AI server and high-tech freight demand alongside fuel-cost pressure. September cargo revenue rose 42.55% year-on-year, but historical revenue does not isolate AI freight volume or pricing.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oct 23, Oct 25</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="98" customHeight="1">
@@ -438,7 +442,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="400" customHeight="1">
+    <row r="6" ht="358" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">04</t>
@@ -453,6 +457,43 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Follow-up: Taipower restores service to over 30,000 affected Yilan accounts by 4 p.m. Oct 25
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 25 Taipower's Yilan branch reported that all more than 30,000 affected household accounts had power restored by 4 p.m. after cross-region repairs. Its Hsinchu branch separately reported 10,886 accounts affected and full restoration by 9 p.m. October 24. These are regional distribution figures, with no disclosed wafer-fab tool downtime or yield losses. Storm damage affected coastal and mountain distribution circuits, including trees touching lines and broken high- and low-voltage conductors. Industrial and fab impacts require site-level electrical records rather than inferred losses from residential restoration numbers. The new October 25 milestone is Yilan's 4 p.m. household restoration completion. The national tally of over 340,000 affected accounts is the previous day's reported backdrop. Hsinchu's complete recovery was a separate October 24 evening update. Taipower cautioned that isolated users on remote line ends may still need to report problems, so full restoration refers to identified affected household accounts. No megawatt load or industrial outage duration was reported. Specific semiconductor tools, data centers and factory downtime or production effects were not disclosed; isolated customer faults may still be reported.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C6" s="6">
+        <v>46320</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-power, UPS and plant monitoring suppliers would review actual voltage dips, storage transfer events and plant alerts. Household restoration totals do not measure tool availability or backup equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="400" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">MViSTA developer targets October cable supplier selection across four Southeast Asian countries
 </t>
           </r>
@@ -466,53 +507,16 @@
           </r>
         </is>
       </c>
-      <c r="C6" s="6">
+      <c r="C7" s="6">
         <v>46317</v>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power, liquid-cooling and metrology suppliers would track the cable tender separately from Vietnam campus feasibility and site power agreements. Landing stations, anchor tenants, power contracts and construction permits are still missing.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="342" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">05</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C7" s="6">
-        <v>46318</v>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="342" customHeight="1">
+    <row r="8" ht="400" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">06</t>
@@ -527,16 +531,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
+            <t xml:space="preserve">Malaysia PM discloses US$50B AI and data-center investment intention, with no approved projects
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 24 in Melaka, Malaysian Prime Minister Anwar Ibrahim said an international investor had conveyed an intended US$50 billion investment across AI, emerging technologies and data centers in Kuching, Sarawak, and Peninsular Malaysia. Singapore's Business Times identified the investor on October 25 as SoftBank's Masayoshi Son, but no SoftBank commitment, approved site, power allocation or construction schedule was published. Large data-center projects depend on server and rack ODMs, UPS and power conversion, cooling, substations and fiber connectivity. Anwar also discussed semiconductor workforce upgrading, without announcing a new wafer-fab project. Bernama recorded Anwar's October 24 public remarks referring to a videoconference held the prior Tuesday. Business Times identified the investor on October 25 and reported that SoftBank had not immediately replied to requests for comment. Neither report included signed agreements or permits. US$50 billion is an attributed multi-sector investment intention, not an approved or disbursed FDI amount. No annual spending profile or site allocation was given, so it cannot be counted as commissioned IT capacity or equipment procurement. Formal investor confirmation, land rights, grid interconnection and load, cooling-water needs, financing, permits and delivery dates are unknown. Location: Kuching, Sarawak, and Peninsular Malaysia are proposed investment regions with no verified site; announcement event held at Hang Jebat Sports Complex, Melaka.</t>
           </r>
         </is>
       </c>
@@ -544,6 +548,117 @@
         <v>46319</v>
       </c>
       <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Power-conversion, UPS, power-quality and liquid-cooling suppliers would verify specific sites, permitted MW load, qualification and purchasing milestones. An aggregate intention without allocation cannot indicate equipment deliveries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="342" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C9" s="6">
+        <v>46318</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="374" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">EVA Air cites sustained high-tech airfreight demand; September cargo revenue rose 42.55%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Speaking in Taipei on October 25, EVA Air president Clay Sun said AI server and other high-tech airfreight demand remained strong through the year, supporting cargo rates, while aviation fuel costs pressured margins. Previously released September cargo revenue was NT$6.167 billion, up 42.55% year on year; it is historical monthly revenue, not October 25 shipment volume. Air cargo transports Taiwan-origin AI servers, racks, semiconductor equipment and high-value electronics. Different cargo types impose distinct weight, space, handling and time constraints; freight revenue cannot be translated directly into equipment production capacity. Management said on October 25 that aviation fuel had reached approximately US$177 per barrel at one point, and that fares and freight rates had been adjusted. September consolidated revenue of NT$20.749 billion and cargo revenue of NT$6.167 billion are earlier reported results, not exclusively AI-related revenue. Cargo-revenue growth reflects shipment volume, rates and product mix, but the report gives no decomposition. US$177 a barrel is a past fuel price referenced by an executive, not a verified spot quote for October 25. Same-day cargo load factors, AI-specific tonnage, long-term customer contracts, fuel-hedging coverage and incremental dedicated freight contracts were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C10" s="6">
+        <v>46320</v>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="342" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C11" s="6">
+        <v>46319</v>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
         </is>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-27 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-25-en.xlsx
+++ b/docs/exports/week-2026-10-25-en.xlsx
@@ -134,21 +134,23 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Rare-earth materials and precision tooling
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">On October 24, ITRI described plans for a rare-earth demo plant by end-2028 and annual output of 500 tonnes by end-2030, aimed at roughly half of Taiwan's demand. Funding, location and qualified material output remain unconfirmed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C3" s="6">
-        <v>46319</v>
+            <t xml:space="preserve">Rare earths, PCB materials and production capacity
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">ITRI's rare-earth demonstration plant remains unfunded and unsited, while Tenghui opened its Thai PCB laminate and prepreg factory on October 26 with small initial shipments. The rare-earth 2030 goal and Thai volume ramp are future targets.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oct 24, Oct 26</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="114" customHeight="1">
@@ -166,26 +168,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Storm recovery, factory power and smart systems
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taipower reported more than 340,000 accounts affected nationwide on October 24, and Yilan declared restoration to over 30,000 affected household accounts by 4 p.m. October 25. The dates and geographies differ, with no fab downtime data. Chunghwa Telecom separately formed an intelligent-vision subsidiary without industrial installation figures.</t>
+            <t xml:space="preserve">Grid restoration, factory AI automation and precision tools
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taipower completed household restoration in Yilan without fab downtime data. Foxconn and NVIDIA reported a 25% scheduling-hour reduction for selected workflows on October 26, and JIMTOF opened in Tokyo with 94 Taiwanese exhibitors according to an association. These metrics measure different activities.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 25</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="130" customHeight="1">
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="118" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -200,22 +202,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Southeast Asian cable tender and Malaysia data-center intentions
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">The MViSTA developer estimates a roughly US$400 million cable with service targeted for late 2028. Malaysia's prime minister separately cited a US$50 billion AI/data-center investment intention on October 24, with media naming SoftBank's Masayoshi Son on October 25. Neither plan supplies approved construction or energization milestones; neither is realized spending.</t>
+            <t xml:space="preserve">Southeast Asia cables, data-center intentions and cross-border power
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">MViSTA's cable remains in tender, Malaysia's prime minister cited a US$50B data-center intention, and Singapore EMA conditionally approved a 1.3GW power import plan for 2035. These are tender, intention and conditional approval stages, not finished infrastructure.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24</t>
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 26</t>
         </is>
       </c>
     </row>
@@ -234,22 +236,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Taiwan optical interconnect and high-tech equipment logistics
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">GSEO and 3M's interconnect collaboration has not published qualified production deliveries. On October 25 EVA Air cited sustained AI server and high-tech freight demand alongside fuel-cost pressure. September cargo revenue rose 42.55% year-on-year, but historical revenue does not isolate AI freight volume or pricing.</t>
+            <t xml:space="preserve">Optical interconnects, cargo and SMT equipment structure
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">GSEO and 3M have not announced qualified EBO production, EVA Air discussed high-tech freight demand on October 25, and Reuters reported potential bids for ASMPT's SMT unit on October 26. Historical bookings, freight revenue and possible deal valuations are not directly comparable.</t>
           </r>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 23, Oct 25</t>
+          <t xml:space="preserve">Oct 23, Oct 25, Oct 26</t>
         </is>
       </c>
     </row>
@@ -268,21 +270,23 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Taiwan-Philippines semiconductor cooperation and 2030 goals
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan's envoy discussed a potential link between Taiwan-Philippines and Luzon economic corridors in Makati on October 24, citing the Philippines' US$110 billion 2030 electronics and semiconductor export goal. No new fab investment approval was announced.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C7" s="6">
-        <v>46319</v>
+            <t xml:space="preserve">Southeast Asian wafer-fab development and semiconductor cooperation
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's envoy discussed Philippine semiconductor corridors and a 2030 electronics export goal. Reuters reported Viettel's Vietnam fab lacked buildings and a finalized DUV order, while Viettel maintained phased progress. No newly commissioned front-end fab was established.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oct 24, Oct 26</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -368,7 +372,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="310" customHeight="1">
+    <row r="4" ht="242" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">02</t>
@@ -383,6 +387,43 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Tenghui opens Thai PCB materials plant and starts small shipments
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Tenghui Electronics opened a roughly 35,000-square-meter copper-clad laminate and prepreg factory at Hi-Tech Industrial Estate in Ayutthaya, Thailand, on October 26, and reported initial shipments. Volume production is targeted by end-2026, with a 15% design-capacity increase planned for 2027; absolute throughput was not disclosed. Copper-clad laminates and prepregs are upstream inputs for server PCBs and automotive electronics. This is Tenghui's first Southeast Asian plant; initial shipments do not establish qualified high-volume output. The company also referenced a previously authorized NT$1.5 billion expansion of its Kunshan, China, plant. That earlier budget is separate from Thailand's factory opening. Thai project capex, monthly shipments, yield and customer qualification remain undisclosed. Location: Hi-Tech Industrial Estate, Ayutthaya, Thailand (operating plant).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C4" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCB process-power and metrology suppliers would verify prepreg line specifications, utilization and customer qualification. Initial shipments do not establish tool acceptance or future procurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="310" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Taipower reports over 340,000 storm-affected accounts and more than 90% restored
 </t>
           </r>
@@ -396,22 +437,22 @@
           </r>
         </is>
       </c>
-      <c r="C4" s="6">
+      <c r="C5" s="6">
         <v>46319</v>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion and industrial power-quality suppliers would separate distribution failure from on-site backup behavior and review insulation protection, UPS transfer and observed voltage events. Without site-level records, tool downtime and lost output cannot be inferred.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="294" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">03</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+    <row r="6" ht="294" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">04</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -433,22 +474,22 @@
           </r>
         </is>
       </c>
-      <c r="C5" s="6">
+      <c r="C6" s="6">
         <v>46317</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial power, machine-vision test and edge compute hardware suppliers would seek camera, server and appliance specifications and site acceptance requirements. No deployment volumes or factory customer contracts were disclosed.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="358" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">04</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+    <row r="7" ht="358" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -470,22 +511,96 @@
           </r>
         </is>
       </c>
-      <c r="C6" s="6">
+      <c r="C7" s="6">
         <v>46320</v>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, UPS and plant monitoring suppliers would review actual voltage dips, storage transfer events and plant alerts. Household restoration totals do not measure tool availability or backup equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="400" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">05</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+    <row r="8" ht="178" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn and NVIDIA report 25% lower scheduling labor hours
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn and NVIDIA reported October 26 that scheduling labor hours fell 25% and molding engineering work fell 50% in selected manufacturing processes. A specified model-training task ran 2.48 times faster on DGX than an older H100 system; cross-factory validation was not disclosed. Applications span SMT, scheduling, automation, metrology and server AI training. NVIDIA cites an H100 comparison and one trillion tokens processed over 12 days; selected workflow outcomes are not factory-wide averages. Test sites, absolute baseline hours and line yield data remain undisclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C8" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metrology and process-power suppliers would verify baseline labor hours and site scope. Results cannot be generalized without controlled samples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="178" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">JIMTOF opens in Tokyo with 94 Taiwan exhibitors, association says
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">JIMTOF opened October 26 at Tokyo Big Sight, running through October 31. Taiwan's machine-tool association reported 94 participating companies covering CNC, metrology and automation; new orders were not disclosed. Precision machinery and controls support industrial automation and semiconductor tool components; exhibiting is not a signed order. Organizer confirms October 26-31 at Tokyo Big Sight; exhibitor number was reported by CNA. Signed deals, qualification and equipment procurement are unknown. Location: Tokyo Big Sight, Tokyo, Japan (exhibition venue).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C9" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Equipment-power and precision metrology suppliers would verify tool specifications and customer acceptance; participation does not prove sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="400" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -507,22 +622,22 @@
           </r>
         </is>
       </c>
-      <c r="C7" s="6">
+      <c r="C10" s="6">
         <v>46317</v>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power, liquid-cooling and metrology suppliers would track the cable tender separately from Vietnam campus feasibility and site power agreements. Landing stations, anchor tenants, power contracts and construction permits are still missing.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="400" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+    <row r="11" ht="400" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -541,117 +656,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">On October 24 in Melaka, Malaysian Prime Minister Anwar Ibrahim said an international investor had conveyed an intended US$50 billion investment across AI, emerging technologies and data centers in Kuching, Sarawak, and Peninsular Malaysia. Singapore's Business Times identified the investor on October 25 as SoftBank's Masayoshi Son, but no SoftBank commitment, approved site, power allocation or construction schedule was published. Large data-center projects depend on server and rack ODMs, UPS and power conversion, cooling, substations and fiber connectivity. Anwar also discussed semiconductor workforce upgrading, without announcing a new wafer-fab project. Bernama recorded Anwar's October 24 public remarks referring to a videoconference held the prior Tuesday. Business Times identified the investor on October 25 and reported that SoftBank had not immediately replied to requests for comment. Neither report included signed agreements or permits. US$50 billion is an attributed multi-sector investment intention, not an approved or disbursed FDI amount. No annual spending profile or site allocation was given, so it cannot be counted as commissioned IT capacity or equipment procurement. Formal investor confirmation, land rights, grid interconnection and load, cooling-water needs, financing, permits and delivery dates are unknown. Location: Kuching, Sarawak, and Peninsular Malaysia are proposed investment regions with no verified site; announcement event held at Hang Jebat Sports Complex, Melaka.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C8" s="6">
-        <v>46319</v>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Power-conversion, UPS, power-quality and liquid-cooling suppliers would verify specific sites, permitted MW load, qualification and purchasing milestones. An aggregate intention without allocation cannot indicate equipment deliveries.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="342" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C9" s="6">
-        <v>46318</v>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="374" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">EVA Air cites sustained high-tech airfreight demand; September cargo revenue rose 42.55%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Speaking in Taipei on October 25, EVA Air president Clay Sun said AI server and other high-tech airfreight demand remained strong through the year, supporting cargo rates, while aviation fuel costs pressured margins. Previously released September cargo revenue was NT$6.167 billion, up 42.55% year on year; it is historical monthly revenue, not October 25 shipment volume. Air cargo transports Taiwan-origin AI servers, racks, semiconductor equipment and high-value electronics. Different cargo types impose distinct weight, space, handling and time constraints; freight revenue cannot be translated directly into equipment production capacity. Management said on October 25 that aviation fuel had reached approximately US$177 per barrel at one point, and that fares and freight rates had been adjusted. September consolidated revenue of NT$20.749 billion and cargo revenue of NT$6.167 billion are earlier reported results, not exclusively AI-related revenue. Cargo-revenue growth reflects shipment volume, rates and product mix, but the report gives no decomposition. US$177 a barrel is a past fuel price referenced by an executive, not a verified spot quote for October 25. Same-day cargo load factors, AI-specific tonnage, long-term customer contracts, fuel-hedging coverage and incremental dedicated freight contracts were not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C10" s="6">
-        <v>46320</v>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="342" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">09</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
           </r>
         </is>
       </c>
@@ -660,7 +664,229 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Power-conversion, UPS, power-quality and liquid-cooling suppliers would verify specific sites, permitted MW load, qualification and purchasing milestones. An aggregate intention without allocation cannot indicate equipment deliveries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="214" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Singapore conditionally approves 1.3GW regional power imports, targeting 2035
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Singapore's EMA conditionally approved Sembcorp Utilities on October 26 to import up to 1.3GW of low-carbon power from a proposed Vietnam-Malaysia-Singapore project, targeting 2035. Offshore wind, solar and storage are proposed sources; approvals, offtake contracts and financing remain pending. The corridor concerns transmission, conversion, storage and data-center power. The 1.3GW figure is approved conditionally, not commissioned capacity. Partners include Petronas, TNB and PTSC, following a May 2025 development agreement. The October 26 approval is conditional, requiring further permits and financing. Routes, capex, tariffs and commissioning timetable remain unconfirmed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C12" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Power conversion and data-center suppliers need transmission specifications, storage designs and offtake terms. No finalized construction or financing plans are available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="342" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C13" s="6">
+        <v>46318</v>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="374" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">EVA Air cites sustained high-tech airfreight demand; September cargo revenue rose 42.55%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Speaking in Taipei on October 25, EVA Air president Clay Sun said AI server and other high-tech airfreight demand remained strong through the year, supporting cargo rates, while aviation fuel costs pressured margins. Previously released September cargo revenue was NT$6.167 billion, up 42.55% year on year; it is historical monthly revenue, not October 25 shipment volume. Air cargo transports Taiwan-origin AI servers, racks, semiconductor equipment and high-value electronics. Different cargo types impose distinct weight, space, handling and time constraints; freight revenue cannot be translated directly into equipment production capacity. Management said on October 25 that aviation fuel had reached approximately US$177 per barrel at one point, and that fares and freight rates had been adjusted. September consolidated revenue of NT$20.749 billion and cargo revenue of NT$6.167 billion are earlier reported results, not exclusively AI-related revenue. Cargo-revenue growth reflects shipment volume, rates and product mix, but the report gives no decomposition. US$177 a barrel is a past fuel price referenced by an executive, not a verified spot quote for October 25. Same-day cargo load factors, AI-specific tonnage, long-term customer contracts, fuel-hedging coverage and incremental dedicated freight contracts were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C14" s="6">
+        <v>46320</v>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="230" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Reuters: Bidding on ASMPT's SMT business continues with no signed sale
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Reuters reported October 26 that IDG Capital was the leading bidder for Singapore-headquartered ASMPT's SMT business, with a potential deal value above US$1 billion, but no agreement finalized. ASMPT's January strategic review considered sale, joint venture, spin-off, listing or retention. SMT equipment covers board printing, placement and inspection for servers, transceivers and electronics. Reported bidding does not establish service or warranty changes. Reuters cited H1 SMT revenue growth of 53.1% to HK$3.87 billion and bookings growth of 87.8% to HK$6.98 billion. Those are historical results; bidder progress is the new claim. No signed agreement, final buyer, price, regulatory filings or workforce plan confirmed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C15" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SMT power, test and service suppliers would track any formal ownership and warranty changes. Reported bidding does not establish a contract transfer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="342" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C16" s="6">
+        <v>46319</v>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="294" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Reuters: Viettel fab lacks buildings and DUV equipment deal remains pending
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Reuters reported October 26 that no buildings have been constructed at Viettel's planned wafer fab outside Hanoi since a January groundbreaking and talks to purchase a DUV lithography tool from ASML remain unresolved. Sources doubt the 2027 trial-production target, whereas Viettel says progress remains in line with its plan. Vietnam already hosts Intel, Amkor and Hana Micron packaging/test sites. Viettel's proposed front-end fab would require lithography, deposition, etch, process power and utilities, distinct from installed packaging capacity. Reuters' site visit and satellite images found no buildings. Authorities previously estimated US$1.3 billion cost, a 2027 trial and full operation by 2030. Viettel says phased progress continues, while ASML has not confirmed a contract. DUV tool type, a signed procurement contract, construction permits, technology partner and validated trial date remain unknown. Location: Planned Viettel wafer fab site on the outskirts of Hanoi, Vietnam (industrial estate not specified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C17" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wafer process-power and metrology suppliers would check signed equipment orders, process partnerships and building permits. Differing site evidence and developer statements leave the 2027 milestone unconfirmed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-28 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-25-en.xlsx
+++ b/docs/exports/week-2026-10-25-en.xlsx
@@ -134,22 +134,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Rare earths, PCB materials and production capacity
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">ITRI's rare-earth demonstration plant remains unfunded and unsited, while Tenghui opened its Thai PCB laminate and prepreg factory on October 26 with small initial shipments. The rare-earth 2030 goal and Thai volume ramp are future targets.</t>
+            <t xml:space="preserve">Memory, electronics materials and rare earths
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">ITRI described a rare-earth demonstration target and Tenghui opened a Thai laminate plant, while Macronix targets H2 2027 new NAND/eMMC output and ESMT reported Q3 earnings. These are planned capacity, opened facilities and realized financial results.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 24, Oct 26</t>
+          <t xml:space="preserve">Oct 24, Oct 26, Oct 27</t>
         </is>
       </c>
     </row>
@@ -168,26 +168,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Grid restoration, factory AI automation and precision tools
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taipower completed household restoration in Yilan without fab downtime data. Foxconn and NVIDIA reported a 25% scheduling-hour reduction for selected workflows on October 26, and JIMTOF opened in Tokyo with 94 Taiwanese exhibitors according to an association. These metrics measure different activities.</t>
+            <t xml:space="preserve">Factory equipment, process metrology and automation
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taipower restored power after a typhoon, Foxconn/NVIDIA reported measured workflow changes and Chunghwa Telecom launched a vision subsidiary. NARLabs/MSS presented a high-NA EUV metrology method and Hongwei reported three years of specialized-lift backlog visibility; these are different metrics.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="118" customHeight="1">
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26, Oct 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="98" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -202,26 +202,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Southeast Asia cables, data-center intentions and cross-border power
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">MViSTA's cable remains in tender, Malaysia's prime minister cited a US$50B data-center intention, and Singapore EMA conditionally approved a 1.3GW power import plan for 2035. These are tender, intention and conditional approval stages, not finished infrastructure.</t>
+            <t xml:space="preserve">Southeast Asian power and data-center infrastructure
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">MViSTA remains in tender, Malaysia's prime minister cited an investment intention, and Singapore EMA granted conditional 1.3GW power-import approval. Delta Thailand approved an intragroup equipment acquisition, none of which independently establishes live data-center capacity.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 26</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="114" customHeight="1">
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 26, Oct 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">04</t>
@@ -236,26 +236,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Optical interconnects, cargo and SMT equipment structure
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">GSEO and 3M have not announced qualified EBO production, EVA Air discussed high-tech freight demand on October 25, and Reuters reported potential bids for ASMPT's SMT unit on October 26. Historical bookings, freight revenue and possible deal valuations are not directly comparable.</t>
+            <t xml:space="preserve">Packaging, optical interconnect and equipment supply
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">GSEO/3M's optical interconnect remains unqualified at volume, EVA Air discussed cargo and ASMPT's SMT sale remains under review. Powertech reports over 30% advanced packaging revenue and CHPT Q3 results reflect probe-card sales, while FOPLP's 2027 ramp is still prospective.</t>
           </r>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 23, Oct 25, Oct 26</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="98" customHeight="1">
+          <t xml:space="preserve">Oct 23, Oct 25, Oct 26, Oct 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="114" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">05</t>
@@ -270,22 +270,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Southeast Asian wafer-fab development and semiconductor cooperation
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan's envoy discussed Philippine semiconductor corridors and a 2030 electronics export goal. Reuters reported Viettel's Vietnam fab lacked buildings and a finalized DUV order, while Viettel maintained phased progress. No newly commissioned front-end fab was established.</t>
+            <t xml:space="preserve">Wafer design, fab development and cross-border cooperation
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Philippine semiconductor corridors remain policy discussions and Reuters reported uncompleted Viettel fab construction and DUV sourcing. Faraday announced a U.S. 2nm GAA design project with Samsung and UMC partnerships; design work, fab building and volume production are separate stages.</t>
           </r>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 24, Oct 26</t>
+          <t xml:space="preserve">Oct 24, Oct 26, Oct 27</t>
         </is>
       </c>
     </row>
@@ -409,7 +409,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="310" customHeight="1">
+    <row r="5" ht="230" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -424,6 +424,80 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Macronix reports NT$24.237B Q3 revenue; new NAND/eMMC output expected H2 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Macronix said on October 27 that Q3 revenue reached NT$24.237 billion, gross margin 70.5% and net profit NT$10.951 billion. Management described more than NT$30 billion in 2026 investment, with added NAND flash and eMMC output emerging only in H2 2027, while NOR expansion is paused and ROM deemphasized. NOR, NAND and eMMC serve industrial, automotive and storage applications. Planned output expansion is distinct from Q3 revenue affected by pricing and product mix. Management said new capacity typically takes more than a year, and near-term sales changes depend on prices; no added monthly wafer-start figure or confirmed tool deliveries were disclosed. Fab allocation, incremental wafer starts, yields and customer order volumes are unavailable.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C5" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Memory process-power and metrology suppliers would seek installed-tool schedules, wafer starts and qualification specifications. A future output target does not establish procurement completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="230" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">04</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Elite Semiconductor Memory reports NT$22.15B sales and NT$10.759B Q3 profit
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Elite Semiconductor Memory announced October 27 Q3 revenue of NT$22.15 billion, gross margin 77.44%, attributable profit NT$10.759 billion and EPS of NT$36.79. Revenue rose 58.8% sequentially and profit around 82%, without a decomposition of pricing, product mix and shipment volume. ESMT sells memory products for a range of applications. Aggregate results do not isolate NAND, DRAM or other product output changes. Q3 gross margin increased 8.74 percentage points sequentially. Jan-Sep revenue of NT$43.363B and profit of NT$18.73B are cumulative figures and not directly comparable with Q3 totals. Original detailed financial statement, category shipments and the separate contribution from price and volume were not independently reviewed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C6" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Memory process-power and testing suppliers would verify wafer starts, product mix and utilization. Higher revenue alone does not establish matching equipment orders or unit shipments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="310" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Taipower reports over 340,000 storm-affected accounts and more than 90% restored
 </t>
           </r>
@@ -437,22 +511,22 @@
           </r>
         </is>
       </c>
-      <c r="C5" s="6">
+      <c r="C7" s="6">
         <v>46319</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion and industrial power-quality suppliers would separate distribution failure from on-site backup behavior and review insulation protection, UPS transfer and observed voltage events. Without site-level records, tool downtime and lost output cannot be inferred.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="294" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">04</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+    <row r="8" ht="294" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -474,22 +548,22 @@
           </r>
         </is>
       </c>
-      <c r="C6" s="6">
+      <c r="C8" s="6">
         <v>46317</v>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial power, machine-vision test and edge compute hardware suppliers would seek camera, server and appliance specifications and site acceptance requirements. No deployment volumes or factory customer contracts were disclosed.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="358" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">05</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
+    <row r="9" ht="358" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -511,22 +585,22 @@
           </r>
         </is>
       </c>
-      <c r="C7" s="6">
+      <c r="C9" s="6">
         <v>46320</v>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, UPS and plant monitoring suppliers would review actual voltage dips, storage transfer events and plant alerts. Household restoration totals do not measure tool availability or backup equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="178" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+    <row r="10" ht="178" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -548,22 +622,22 @@
           </r>
         </is>
       </c>
-      <c r="C8" s="6">
+      <c r="C10" s="6">
         <v>46321</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Metrology and process-power suppliers would verify baseline labor hours and site scope. Results cannot be generalized without controlled samples.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="178" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+    <row r="11" ht="178" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -585,22 +659,96 @@
           </r>
         </is>
       </c>
-      <c r="C9" s="6">
+      <c r="C11" s="6">
         <v>46321</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Equipment-power and precision metrology suppliers would verify tool specifications and customer acceptance; participation does not prove sales.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="400" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+    <row r="12" ht="262" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">NARLabs and MSS report high-NA EUV resist cross-section metrology technique
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">NARLabs announced October 27 that its instrumentation center and Materials Analysis Technology Inc. (MSS) developed a coating approach to stabilize high-NA EUV metal-oxide-resist nanostructures for subsequent wafer cross-section analysis. NARLabs says it helped MSS enter major semiconductor suppliers' process chains, without customer acceptance, yield or deployment volumes. High-NA EUV metal-oxide-resist patterns require structural preservation during cross-section sample preparation, linking advanced lithography to metrology and microscopy. NARLabs describes stabilizing fragile patterned structures with coating prior to analysis. The disclosed research milestone is not evidence of a qualified high-volume manufacturing node. Comparative defect rates, tested resolution, fab qualification dates and commercial metrology orders were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C12" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-metrology, power and analysis-tool suppliers would examine material compatibility, specimen reproducibility and qualification. Research success does not establish volume tool contracts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="246" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Hongwei says specialized industrial lift orders now provide three years of visibility
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 27, Hongwei Electric said its backlog for heavy-duty, cleanroom and automated material-handling lifts now offers three years of visibility, with orders on hand doubling versus 2025. It described semiconductor-related shipments as roughly 59% of the relevant mix, without disclosing absolute contract value or customer site details. Cleanroom, heavy-load and explosion-proof lifts support factory logistics and utilities, not front-end lithography or process equipment. Management said orders-to-shipments remained above one and reported sales to semiconductor and testing-related customers; three-year backlog visibility is a company estimate, not realized revenue. Absolute backlog units, contract values, delivery schedule and named project sites were not disclosed or independently verified.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C13" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial power and material-handling suppliers would seek delivery sites, load ratings and acceptance milestones. Backlog visibility is not recognized revenue or evidence of wafer-fab commissioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="400" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -622,22 +770,22 @@
           </r>
         </is>
       </c>
-      <c r="C10" s="6">
+      <c r="C14" s="6">
         <v>46317</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power, liquid-cooling and metrology suppliers would track the cable tender separately from Vietnam campus feasibility and site power agreements. Landing stations, anchor tenants, power contracts and construction permits are still missing.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="400" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">09</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+    <row r="15" ht="400" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -659,22 +807,22 @@
           </r>
         </is>
       </c>
-      <c r="C11" s="6">
+      <c r="C15" s="6">
         <v>46319</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion, UPS, power-quality and liquid-cooling suppliers would verify specific sites, permitted MW load, qualification and purchasing milestones. An aggregate intention without allocation cannot indicate equipment deliveries.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="214" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+    <row r="16" ht="214" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -696,22 +844,59 @@
           </r>
         </is>
       </c>
-      <c r="C12" s="6">
+      <c r="C16" s="6">
         <v>46321</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power conversion and data-center suppliers need transmission specifications, storage designs and offtake terms. No finalized construction or financing plans are available.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="342" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+    <row r="17" ht="278" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Delta Thailand plans US$34.5M equipment purchase from Singapore affiliate
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Delta Electronics announced October 27 that its Thai subsidiary DET approved acquiring roughly US$34.5 million of operating equipment from fellow group company DEIL-SG in Singapore to support smart-factory manufacturing. It is a related-party asset transaction, not proof of incremental foreign investment or completed commissioning. Intercompany equipment transfers can concern line automation and production allocation. The disclosure only calls the assets operating equipment, without model or line detail. CNA reported the company's October 27 material disclosure: DET's board approved an approximately US$34.5M related-party acquisition from the group's Singapore unit, with negotiated terms and wire payment. Equipment list, plant location, carrying value, installation timing, capacity changes and settlement date remain undisclosed. Location: DET Thailand (installation site undisclosed); seller is a group affiliate in Singapore.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C17" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart-factory power and test suppliers would check equipment type, whether transferred or newly built, and acceptance status. An intercompany book transaction cannot establish incremental production capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="342" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -733,22 +918,22 @@
           </r>
         </is>
       </c>
-      <c r="C13" s="6">
+      <c r="C18" s="6">
         <v>46318</v>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="374" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
+    <row r="19" ht="374" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -770,22 +955,22 @@
           </r>
         </is>
       </c>
-      <c r="C14" s="6">
+      <c r="C19" s="6">
         <v>46320</v>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="230" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+    <row r="20" ht="230" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -807,22 +992,96 @@
           </r>
         </is>
       </c>
-      <c r="C15" s="6">
+      <c r="C20" s="6">
         <v>46321</v>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">SMT power, test and service suppliers would track any formal ownership and warranty changes. Reported bidding does not establish a contract transfer.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="342" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+    <row r="21" ht="262" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Powertech says advanced packaging exceeds 30% of revenue and utilization tops 90%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Powertech Technology reported October 27 third-quarter revenue of NT$25.334 billion, 24% gross margin and NT$2.612 billion in profit attributable to shareholders. It said advanced packaging now exceeds 30% of group revenue and packaging/test utilization topped 90% in Q3; FOPLP qualification, the 2027 production target and its Singapore investment remain pending. The company serves DRAM, NAND/eSSD and logic packaging, with planned FOPLP, FCBGA, heterogeneous integration and optical engines for CPO. These product types cannot be counted as one commissioned capacity. Large-die FCBGA entered production in Q3 according to management, with larger packages slated for Q4. FOPLP remains a 2027 target, and potential alliances with foundries are not signed agreements. FOPLP customer acceptance, absolute monthly capacity, Singapore investment size and shipment dates were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C21" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Packaging tool, test-power and metrology suppliers would check qualified package sizes, line requirements and actual delivery milestones. Q3 utilization and future expansion are separate measures, not equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="230" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">CHPT reports NT$1.905B Q3 sales and NT$551M profit; probe cards lead mix
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">CHPT's board approved October 27 Q3 results showing NT$1.905 billion revenue, up 53.4% YoY, and NT$551 million attributable profit, up 100% YoY. Wafer probe cards accounted for 71% of Jan-Sep revenue and IC load boards for 21%; next-generation customer qualification data is not public. Wafer probe cards and IC load boards support wafer sorting and package test for memory and AI ASICs. Revenue mix is not production quantity. Its primary release reports 57.3% Q3 gross margin and roughly 35% operating margin, citing demand for customized AI testing interfaces. It gives growth rates without every absolute prior-year base. Next-generation probe-card customer roster, utilization, qualification times and new tool investments were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C22" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-frequency test-power and probe-card suppliers would seek channel-level signal/power-integrity specifications and qualification timelines. Sales mix cannot quantify tester procurement or throughput.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="342" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -844,22 +1103,22 @@
           </r>
         </is>
       </c>
-      <c r="C16" s="6">
+      <c r="C23" s="6">
         <v>46319</v>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="294" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
+    <row r="24" ht="294" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -881,12 +1140,49 @@
           </r>
         </is>
       </c>
-      <c r="C17" s="6">
+      <c r="C24" s="6">
         <v>46321</v>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Wafer process-power and metrology suppliers would check signed equipment orders, process partnerships and building permits. Differing site evidence and developer statements leave the 2027 milestone unconfirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="246" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Faraday secures Samsung 2nm GAA design project, targets first revenue in H1 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 27, Faraday Technology announced a U.S. cloud AI chip non-recurring engineering project using Samsung's 2nm GAA foundry, with UMC and memory partners. Management described project value in the tens of millions of U.S. dollars and expects initial revenue recognition in H1 2027, without a precise contract value or qualified production date. The design project requires advanced-node IP and coordination across foundry and memory partners. UMC's participation does not make it the 2nm wafer foundry. Q3 revenue was NT$3.664B, gross margin 42.5% and attributable profit NT$279M. Management attributed margin changes partly to product mix and profit changes partly to non-operating valuation gains. Customer identity, package technology, exact NRE timing and chip shipment volumes were not given.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C25" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wafer process-power and advanced packaging test suppliers would verify actual foundry, package interface and qualification milestones. NRE contract value is not wafer manufacturing or equipment spending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-29 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-25-en.xlsx
+++ b/docs/exports/week-2026-10-25-en.xlsx
@@ -134,22 +134,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Memory, electronics materials and rare earths
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">ITRI described a rare-earth demonstration target and Tenghui opened a Thai laminate plant, while Macronix targets H2 2027 new NAND/eMMC output and ESMT reported Q3 earnings. These are planned capacity, opened facilities and realized financial results.</t>
+            <t xml:space="preserve">Memory modules, materials and high-speed chips
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">ITRI presented a rare-earth plan, Tenghui's Thai CCL plant began small shipments and Macronix memory expansion targets 2027. TeamGroup plans Q2 2027 module production while Parade guided lower Q4 interface-chip revenue; actuals, plans and forecasts have different statuses.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 24, Oct 26, Oct 27</t>
+          <t xml:space="preserve">Oct 24, Oct 26, Oct 27, Oct 28</t>
         </is>
       </c>
     </row>
@@ -168,26 +168,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Factory equipment, process metrology and automation
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taipower restored power after a typhoon, Foxconn/NVIDIA reported measured workflow changes and Chunghwa Telecom launched a vision subsidiary. NARLabs/MSS presented a high-NA EUV metrology method and Hongwei reported three years of specialized-lift backlog visibility; these are different metrics.</t>
+            <t xml:space="preserve">Wafer testing, factory automation and precision tools
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Grid restoration, Foxconn's AI manufacturing measurements and a NARLabs/MSS high-NA EUV metrology method represent separate stages. CHPT reported probe-card results and a 2027 capacity target on October 28, while Jin-An opened its Longtan factory; absolute throughput and deliveries remain distinct.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26, Oct 27</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="98" customHeight="1">
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26, Oct 27, Oct 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="134" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -202,26 +202,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Southeast Asian power and data-center infrastructure
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">MViSTA remains in tender, Malaysia's prime minister cited an investment intention, and Singapore EMA granted conditional 1.3GW power-import approval. Delta Thailand approved an intragroup equipment acquisition, none of which independently establishes live data-center capacity.</t>
+            <t xml:space="preserve">Power and data-center infrastructure across Taiwan and Southeast Asia
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">MViSTA remains in tender, Malaysia's US$50B intention lacks approved projects and Singapore granted conditional power-import approval. Delta published Q3 results and Chief Telecom described data-center revenue and an LY2 occupancy goal; financial results, intentions and energized capacity are different measures.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 26, Oct 27</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98" customHeight="1">
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 26, Oct 27, Oct 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="114" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">04</t>
@@ -236,22 +236,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Packaging, optical interconnect and equipment supply
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">GSEO/3M's optical interconnect remains unqualified at volume, EVA Air discussed cargo and ASMPT's SMT sale remains under review. Powertech reports over 30% advanced packaging revenue and CHPT Q3 results reflect probe-card sales, while FOPLP's 2027 ramp is still prospective.</t>
+            <t xml:space="preserve">Advanced packaging, optics and electronics test equipment
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">GSEO and 3M's optical interconnect has no published customer volume qualification, while Powertech's advanced packaging share exceeds 30% but FOPLP awaits qualification. ASMPT's SMT divestiture remains unsigned and WIN reported Q3 results and a photodiode ramp on October 28, with future deliveries unconfirmed.</t>
           </r>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 23, Oct 25, Oct 26, Oct 27</t>
+          <t xml:space="preserve">Oct 23, Oct 25, Oct 26, Oct 27, Oct 28</t>
         </is>
       </c>
     </row>
@@ -270,22 +270,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Wafer design, fab development and cross-border cooperation
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Philippine semiconductor corridors remain policy discussions and Reuters reported uncompleted Viettel fab construction and DUV sourcing. Faraday announced a U.S. 2nm GAA design project with Samsung and UMC partnerships; design work, fab building and volume production are separate stages.</t>
+            <t xml:space="preserve">Wafer fabrication, regional cooperation and chip controls
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Philippine semiconductor corridors remain policy discussions, Reuters reported incomplete Viettel fab and DUV milestones, and Faraday disclosed a 2nm design project. UMC authorized about US$3.2B extra expansion on October 28; Malaysian customs separately disclosed an October 15 AI-server seizure, with distinct approval and enforcement dates.</t>
           </r>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 24, Oct 26, Oct 27</t>
+          <t xml:space="preserve">Oct 15, Oct 24, Oct 26, Oct 27, Oct 28</t>
         </is>
       </c>
     </row>
@@ -483,7 +483,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="310" customHeight="1">
+    <row r="7" ht="262" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">05</t>
@@ -498,6 +498,80 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">TeamGroup plans New Taipei factory launch in Q2 2027 with 50% capacity increase
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 28, TeamGroup described purchasing an approximately 1,000-ping facility in New Taipei City, targeting automation installation in Q1 2027 and production in Q2, with roughly 50% additional capacity. Q3 revenue was NT$10.139 billion and EPS NT$37.19; inconsistent net-profit figures within the same report are omitted pending reconciliation. TeamGroup makes DRAM and SSD modules for enterprise, industrial and consumer systems. The new factory expands module assembly/test, not upstream DRAM wafer capacity. The company also reorganized business units and acquired about 700 ping of office space. The 50% target lacks a published absolute monthly-output base or equipment capex. Exact location, transaction value, tool orders, qualified module output and the conflicting net-profit figure remain unresolved. Location: New Taipei City, Taiwan (acquired facility; exact address not disclosed).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C7" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Memory module test-power and automation suppliers would verify test flow, utilization and qualification; 50% is a projected capacity uplift, not installed output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="230" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">06</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Parade expects Q4 revenue down 20% to 27% as PC costs weigh on interface chips
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Parade Technologies guided October 28 for Q4 revenue of US$95 million to US$105 million, down 20% to 27% sequentially, versus Q3 revenue near US$130 million and a 40.29% gross margin. Management linked PC softness to DRAM and manufacturing cost increases; Q4 margin guidance of 41% to 45% is a forecast. High-speed interface chips support PCs, displays and data links through foundry and test supply chains. Volume and pricing are affected by multiple factors, not solely DRAM costs. Management reported foundry and test cost increases and planned pricing changes. Q4 figures are ranges rather than firm orders. Named PC customer volumes, pass-through percentages and actual Q4 shipped mix remain undisclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C8" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Foundry process-power and test suppliers would distinguish current interface-chip shipments from Q4 guidance and verify actual demand/mix. Pricing pass-through needs later earnings confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="310" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Taipower reports over 340,000 storm-affected accounts and more than 90% restored
 </t>
           </r>
@@ -511,22 +585,22 @@
           </r>
         </is>
       </c>
-      <c r="C7" s="6">
+      <c r="C9" s="6">
         <v>46319</v>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion and industrial power-quality suppliers would separate distribution failure from on-site backup behavior and review insulation protection, UPS transfer and observed voltage events. Without site-level records, tool downtime and lost output cannot be inferred.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="294" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+    <row r="10" ht="294" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -548,22 +622,22 @@
           </r>
         </is>
       </c>
-      <c r="C8" s="6">
+      <c r="C10" s="6">
         <v>46317</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial power, machine-vision test and edge compute hardware suppliers would seek camera, server and appliance specifications and site acceptance requirements. No deployment volumes or factory customer contracts were disclosed.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="358" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+    <row r="11" ht="358" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -585,22 +659,22 @@
           </r>
         </is>
       </c>
-      <c r="C9" s="6">
+      <c r="C11" s="6">
         <v>46320</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, UPS and plant monitoring suppliers would review actual voltage dips, storage transfer events and plant alerts. Household restoration totals do not measure tool availability or backup equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="178" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+    <row r="12" ht="178" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -622,22 +696,22 @@
           </r>
         </is>
       </c>
-      <c r="C10" s="6">
+      <c r="C12" s="6">
         <v>46321</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Metrology and process-power suppliers would verify baseline labor hours and site scope. Results cannot be generalized without controlled samples.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="178" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">09</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+    <row r="13" ht="178" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -659,22 +733,22 @@
           </r>
         </is>
       </c>
-      <c r="C11" s="6">
+      <c r="C13" s="6">
         <v>46321</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Equipment-power and precision metrology suppliers would verify tool specifications and customer acceptance; participation does not prove sales.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="262" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+    <row r="14" ht="262" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -696,22 +770,22 @@
           </r>
         </is>
       </c>
-      <c r="C12" s="6">
+      <c r="C14" s="6">
         <v>46322</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-metrology, power and analysis-tool suppliers would examine material compatibility, specimen reproducibility and qualification. Research success does not establish volume tool contracts.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="246" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
+    <row r="15" ht="246" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -733,22 +807,96 @@
           </r>
         </is>
       </c>
-      <c r="C13" s="6">
+      <c r="C15" s="6">
         <v>46322</v>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial power and material-handling suppliers would seek delivery sites, load ratings and acceptance milestones. Backlog visibility is not recognized revenue or evidence of wafer-fab commissioning.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="400" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
+    <row r="16" ht="246" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Follow-up: CHPT reports nearly NT$400M Q3 advanced probe-card sales and 3x capacity target
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At an October 28 briefing, CHPT said advanced probe cards contributed nearly NT$400 million or 21% of Q3 revenue, while HPC products represented 65.9%. Capacity had doubled relative to end-2025 by August, with a threefold level targeted for Q1 2027, adding operational detail to the previous day's earnings. Probe cards, wafer test boards and high-power burn-in systems serve GPUs, TPUs, ASICs and CPO testing. Signal, power-integrity and temperature requirements differ by product. Management expects engineering CPU probe-card samples in November and targets volume production in 2027; CPO test interface talks involve more than five firms. These are stated qualification and commercial milestones, not completed acceptance. Absolute throughput, channel counts, accepted customers and high-power burn-in board volumes remain undisclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C16" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test-power, prober and burn-in suppliers would verify power density, channel requirements and qualification dates. A capacity multiple without absolute unit throughput cannot determine equipment volumes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="310" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Jin-An Machinery opens Longtan plant for ice-storage cooling and industrial unmanned systems
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">I-Mei affiliate Jin-An Machinery opened a new manufacturing building in Longtan, Taoyuan on October 28, following investment above NT$1 billion. The facility plans to make more than 20 off-peak ice-storage cooling systems for group factories; management claims a 25% to 30% reduction in peak electricity draw at an existing Longtan site, not a universal efficiency result. Ice-storage cooling shifts HVAC electricity loads from daytime to off-peak hours, rather than directly reducing chip-cooling load or total kWh. Unmanned systems and environmental tests are a separate line of work. The facility houses freeze-drying, thermal-storage and unmanned-system production. The above-NT$1B figure is a company-stated project total without tool/facility breakdown; 20-plus cooling systems are prospective production. Construction periods, individual system kW ratings, measured kWh and external customer acceptance counts are unavailable. Location: Longtan District, Taoyuan City, Taiwan, Jin-An manufacturing building (opened site, street address not verified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C17" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial cooling, drives and power-controls suppliers would verify thermal-storage size, load profiles and peak demand calculations. A single site's reduction is not a universal data-center efficiency result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="400" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -770,22 +918,22 @@
           </r>
         </is>
       </c>
-      <c r="C14" s="6">
+      <c r="C18" s="6">
         <v>46317</v>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power, liquid-cooling and metrology suppliers would track the cable tender separately from Vietnam campus feasibility and site power agreements. Landing stations, anchor tenants, power contracts and construction permits are still missing.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="400" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+    <row r="19" ht="400" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -807,22 +955,22 @@
           </r>
         </is>
       </c>
-      <c r="C15" s="6">
+      <c r="C19" s="6">
         <v>46319</v>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion, UPS, power-quality and liquid-cooling suppliers would verify specific sites, permitted MW load, qualification and purchasing milestones. An aggregate intention without allocation cannot indicate equipment deliveries.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="214" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+    <row r="20" ht="214" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -841,154 +989,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">Singapore's EMA conditionally approved Sembcorp Utilities on October 26 to import up to 1.3GW of low-carbon power from a proposed Vietnam-Malaysia-Singapore project, targeting 2035. Offshore wind, solar and storage are proposed sources; approvals, offtake contracts and financing remain pending. The corridor concerns transmission, conversion, storage and data-center power. The 1.3GW figure is approved conditionally, not commissioned capacity. Partners include Petronas, TNB and PTSC, following a May 2025 development agreement. The October 26 approval is conditional, requiring further permits and financing. Routes, capex, tariffs and commissioning timetable remain unconfirmed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C16" s="6">
-        <v>46321</v>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Power conversion and data-center suppliers need transmission specifications, storage designs and offtake terms. No finalized construction or financing plans are available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="278" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Delta Thailand plans US$34.5M equipment purchase from Singapore affiliate
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Delta Electronics announced October 27 that its Thai subsidiary DET approved acquiring roughly US$34.5 million of operating equipment from fellow group company DEIL-SG in Singapore to support smart-factory manufacturing. It is a related-party asset transaction, not proof of incremental foreign investment or completed commissioning. Intercompany equipment transfers can concern line automation and production allocation. The disclosure only calls the assets operating equipment, without model or line detail. CNA reported the company's October 27 material disclosure: DET's board approved an approximately US$34.5M related-party acquisition from the group's Singapore unit, with negotiated terms and wire payment. Equipment list, plant location, carrying value, installation timing, capacity changes and settlement date remain undisclosed. Location: DET Thailand (installation site undisclosed); seller is a group affiliate in Singapore.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C17" s="6">
-        <v>46322</v>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Smart-factory power and test suppliers would check equipment type, whether transferred or newly built, and acceptance status. An intercompany book transaction cannot establish incremental production capacity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="342" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C18" s="6">
-        <v>46318</v>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="374" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">EVA Air cites sustained high-tech airfreight demand; September cargo revenue rose 42.55%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Speaking in Taipei on October 25, EVA Air president Clay Sun said AI server and other high-tech airfreight demand remained strong through the year, supporting cargo rates, while aviation fuel costs pressured margins. Previously released September cargo revenue was NT$6.167 billion, up 42.55% year on year; it is historical monthly revenue, not October 25 shipment volume. Air cargo transports Taiwan-origin AI servers, racks, semiconductor equipment and high-value electronics. Different cargo types impose distinct weight, space, handling and time constraints; freight revenue cannot be translated directly into equipment production capacity. Management said on October 25 that aviation fuel had reached approximately US$177 per barrel at one point, and that fares and freight rates had been adjusted. September consolidated revenue of NT$20.749 billion and cargo revenue of NT$6.167 billion are earlier reported results, not exclusively AI-related revenue. Cargo-revenue growth reflects shipment volume, rates and product mix, but the report gives no decomposition. US$177 a barrel is a past fuel price referenced by an executive, not a verified spot quote for October 25. Same-day cargo load factors, AI-specific tonnage, long-term customer contracts, fuel-hedging coverage and incremental dedicated freight contracts were not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C19" s="6">
-        <v>46320</v>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="230" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Reuters: Bidding on ASMPT's SMT business continues with no signed sale
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Reuters reported October 26 that IDG Capital was the leading bidder for Singapore-headquartered ASMPT's SMT business, with a potential deal value above US$1 billion, but no agreement finalized. ASMPT's January strategic review considered sale, joint venture, spin-off, listing or retention. SMT equipment covers board printing, placement and inspection for servers, transceivers and electronics. Reported bidding does not establish service or warranty changes. Reuters cited H1 SMT revenue growth of 53.1% to HK$3.87 billion and bookings growth of 87.8% to HK$6.98 billion. Those are historical results; bidder progress is the new claim. No signed agreement, final buyer, price, regulatory filings or workforce plan confirmed.</t>
           </r>
         </is>
       </c>
@@ -997,11 +997,11 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMT power, test and service suppliers would track any formal ownership and warranty changes. Reported bidding does not establish a contract transfer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="262" customHeight="1">
+          <t xml:space="preserve">Power conversion and data-center suppliers need transmission specifications, storage designs and offtake terms. No finalized construction or financing plans are available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="278" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">19</t>
@@ -1016,16 +1016,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Powertech says advanced packaging exceeds 30% of revenue and utilization tops 90%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Powertech Technology reported October 27 third-quarter revenue of NT$25.334 billion, 24% gross margin and NT$2.612 billion in profit attributable to shareholders. It said advanced packaging now exceeds 30% of group revenue and packaging/test utilization topped 90% in Q3; FOPLP qualification, the 2027 production target and its Singapore investment remain pending. The company serves DRAM, NAND/eSSD and logic packaging, with planned FOPLP, FCBGA, heterogeneous integration and optical engines for CPO. These product types cannot be counted as one commissioned capacity. Large-die FCBGA entered production in Q3 according to management, with larger packages slated for Q4. FOPLP remains a 2027 target, and potential alliances with foundries are not signed agreements. FOPLP customer acceptance, absolute monthly capacity, Singapore investment size and shipment dates were not disclosed.</t>
+            <t xml:space="preserve">Delta Thailand plans US$34.5M equipment purchase from Singapore affiliate
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Delta Electronics announced October 27 that its Thai subsidiary DET approved acquiring roughly US$34.5 million of operating equipment from fellow group company DEIL-SG in Singapore to support smart-factory manufacturing. It is a related-party asset transaction, not proof of incremental foreign investment or completed commissioning. Intercompany equipment transfers can concern line automation and production allocation. The disclosure only calls the assets operating equipment, without model or line detail. CNA reported the company's October 27 material disclosure: DET's board approved an approximately US$34.5M related-party acquisition from the group's Singapore unit, with negotiated terms and wire payment. Equipment list, plant location, carrying value, installation timing, capacity changes and settlement date remain undisclosed. Location: DET Thailand (installation site undisclosed); seller is a group affiliate in Singapore.</t>
           </r>
         </is>
       </c>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Packaging tool, test-power and metrology suppliers would check qualified package sizes, line requirements and actual delivery milestones. Q3 utilization and future expansion are separate measures, not equipment orders.</t>
+          <t xml:space="preserve">Smart-factory power and test suppliers would check equipment type, whether transferred or newly built, and acceptance status. An intercompany book transaction cannot establish incremental production capacity.</t>
         </is>
       </c>
     </row>
@@ -1053,6 +1053,228 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Delta Electronics Q3 revenue reaches NT$197.059B; attributable profit NT$23.495B
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Delta Electronics released October 28 Q3 results: NT$197.059 billion revenue, NT$23.495 billion attributable profit and EPS of NT$9.04. Sales rose roughly 31% year on year while profit declined 6.5% sequentially; an October 29 investor call has yet to provide updated power and cooling guidance. Delta's consolidated business spans server power, data-center infrastructure, thermal systems and automation. Group revenue does not measure AI rack power alone. Q3 gross margin was 34.08%, down 0.79 percentage points year over year, and attributable profit rose 26.3% YoY but fell 6.5% QoQ. The next day's investor guidance is not yet available. Separate HVDC, liquid-cooling and rack power revenue/profit and October 29 guidance are unavailable.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C22" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Power and industrial metrology suppliers would separate group results from actual delivery of data-center modules and monitor later product qualification disclosures. Consolidated sales alone cannot quantify new rack deployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="262" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Chief Telecom reports NT$1.077B Q3 revenue and targets 80% LY2 occupancy by year-end
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Chief Telecom reported October 28 Q3 revenue of NT$1.077 billion, gross margin of 51.5% and net income NT$332 million. Management targets 80% occupancy at LY2 by year-end; the Huwei AI data-center project broke ground October 20 and aims for H2 2028 operation, with no new commissioned IT load or rack count disclosed. Data-center tenancy relates to UPS, electricity, cooling and interconnect. Occupancy is not equal to IT power loading or GPU utilization. Management said LY2 depreciation is now fully reflected, with Q3 gross margin above the first-half 48.55% level. An 80% year-end occupancy is a target, not the occupancy verified on October 28. Current occupancy, total racks, energized MW, cooling density and Huwei capacity are not disclosed. Location: LY2 operating data center in Taipei, Taiwan; separate planned AI data-center project site in Huwei, Yunlin County.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C23" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UPS, power and liquid-cooling suppliers would verify the occupancy denominator, energized racks and power per cabinet. An 80% tenancy goal is not an equipment purchase count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="342" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C24" s="6">
+        <v>46318</v>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="374" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">EVA Air cites sustained high-tech airfreight demand; September cargo revenue rose 42.55%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Speaking in Taipei on October 25, EVA Air president Clay Sun said AI server and other high-tech airfreight demand remained strong through the year, supporting cargo rates, while aviation fuel costs pressured margins. Previously released September cargo revenue was NT$6.167 billion, up 42.55% year on year; it is historical monthly revenue, not October 25 shipment volume. Air cargo transports Taiwan-origin AI servers, racks, semiconductor equipment and high-value electronics. Different cargo types impose distinct weight, space, handling and time constraints; freight revenue cannot be translated directly into equipment production capacity. Management said on October 25 that aviation fuel had reached approximately US$177 per barrel at one point, and that fares and freight rates had been adjusted. September consolidated revenue of NT$20.749 billion and cargo revenue of NT$6.167 billion are earlier reported results, not exclusively AI-related revenue. Cargo-revenue growth reflects shipment volume, rates and product mix, but the report gives no decomposition. US$177 a barrel is a past fuel price referenced by an executive, not a verified spot quote for October 25. Same-day cargo load factors, AI-specific tonnage, long-term customer contracts, fuel-hedging coverage and incremental dedicated freight contracts were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C25" s="6">
+        <v>46320</v>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="230" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Reuters: Bidding on ASMPT's SMT business continues with no signed sale
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Reuters reported October 26 that IDG Capital was the leading bidder for Singapore-headquartered ASMPT's SMT business, with a potential deal value above US$1 billion, but no agreement finalized. ASMPT's January strategic review considered sale, joint venture, spin-off, listing or retention. SMT equipment covers board printing, placement and inspection for servers, transceivers and electronics. Reported bidding does not establish service or warranty changes. Reuters cited H1 SMT revenue growth of 53.1% to HK$3.87 billion and bookings growth of 87.8% to HK$6.98 billion. Those are historical results; bidder progress is the new claim. No signed agreement, final buyer, price, regulatory filings or workforce plan confirmed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C26" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SMT power, test and service suppliers would track any formal ownership and warranty changes. Reported bidding does not establish a contract transfer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="262" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Powertech says advanced packaging exceeds 30% of revenue and utilization tops 90%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Powertech Technology reported October 27 third-quarter revenue of NT$25.334 billion, 24% gross margin and NT$2.612 billion in profit attributable to shareholders. It said advanced packaging now exceeds 30% of group revenue and packaging/test utilization topped 90% in Q3; FOPLP qualification, the 2027 production target and its Singapore investment remain pending. The company serves DRAM, NAND/eSSD and logic packaging, with planned FOPLP, FCBGA, heterogeneous integration and optical engines for CPO. These product types cannot be counted as one commissioned capacity. Large-die FCBGA entered production in Q3 according to management, with larger packages slated for Q4. FOPLP remains a 2027 target, and potential alliances with foundries are not signed agreements. FOPLP customer acceptance, absolute monthly capacity, Singapore investment size and shipment dates were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C27" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Packaging tool, test-power and metrology suppliers would check qualified package sizes, line requirements and actual delivery milestones. Q3 utilization and future expansion are separate measures, not equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="230" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">CHPT reports NT$1.905B Q3 sales and NT$551M profit; probe cards lead mix
 </t>
           </r>
@@ -1066,22 +1288,59 @@
           </r>
         </is>
       </c>
-      <c r="C22" s="6">
+      <c r="C28" s="6">
         <v>46322</v>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">High-frequency test-power and probe-card suppliers would seek channel-level signal/power-integrity specifications and qualification timelines. Sales mix cannot quantify tester procurement or throughput.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="342" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">21</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
+    <row r="29" ht="246" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">27</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">WIN Semiconductors Q3 sales reach NT$5.859B; photodiode ramp ongoing
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">WIN Semiconductors announced October 28 Q3 revenue of NT$5.859 billion, gross margin 37.4% and attributable profit of NT$1.93 billion. Optical receiver photodiodes remain in early production ramp, with management pointing to larger-scale shipments in 2028; application-level volume was not reported. WIN's GaAs RF and receiver products serve satellite links, optical communications and data-center modules. Revenue growth is not evidence of new wafer-fab commissioning. Management said gross margin rose 9.2 percentage points from Q2 and profit increased around 98% sequentially. Q4 revenue guidance is low-single-digit sequential growth amid mixed handset demand. PD monthly shipments, yields, qualified customers and planned 2028 capacity allocations were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C29" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RF process-power and optical metrology suppliers would verify PD yields and receiver test bandwidth. Future volume projections cannot be inferred from consolidated profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="342" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1103,22 +1362,22 @@
           </r>
         </is>
       </c>
-      <c r="C23" s="6">
+      <c r="C30" s="6">
         <v>46319</v>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="294" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
+    <row r="31" ht="294" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1140,22 +1399,22 @@
           </r>
         </is>
       </c>
-      <c r="C24" s="6">
+      <c r="C31" s="6">
         <v>46321</v>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Wafer process-power and metrology suppliers would check signed equipment orders, process partnerships and building permits. Differing site evidence and developer statements leave the 2027 milestone unconfirmed.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="246" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
+    <row r="32" ht="246" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1177,12 +1436,86 @@
           </r>
         </is>
       </c>
-      <c r="C25" s="6">
+      <c r="C32" s="6">
         <v>46322</v>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Wafer process-power and advanced packaging test suppliers would verify actual foundry, package interface and qualification milestones. NRE contract value is not wafer manufacturing or equipment spending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="310" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">UMC approves approximately US$3.2B additional capacity budget for Singapore and Tainan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 28, UMC's board approved around US$3.2 billion of additional expansion budget, intended to accelerate its Singapore and Tainan capacity plans, with no individual ramp dates. Q3 revenue was NT$74.24 billion, gross margin 34%, 12-inch-equivalent shipments over 1.2 million wafers and utilization 92%. The foundry serves mature and specialty nodes including 22/28nm technologies for power management, connectivity, silicon photonics and industrial controls. Board-authorized funding is not commissioned equipment or cash spent. UMC described US$2 billion 2026 capex separately from the new authorization. Guidance calls for Q4 shipment growth of 1% to 3% and utilization of 91% to 93%; 2027 blended ASP growth of 10% is a management expectation, not realized pricing. Site-by-site spending, tool awards, additional wafer starts, construction and commissioning dates are unknown; ASP and AI mix statements are forecasts. Location: Tainan Science Park, Taiwan, and Singapore facilities (regions for expansion; specific new building sites unspecified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C33" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-power, metrology and packaging tool suppliers would verify equipment specifications and procurement schedules separately for Singapore and Tainan. Authorization and current utilization do not establish tool delivery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="278" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Malaysia customs reports seizure of 30 servers containing AI chips valued near MYR49.5M
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 28, Malaysian customs disclosed that it intercepted 30 servers carrying advanced AI chips at Kuala Lumpur International Airport's free trade zone on October 15, estimating their value at MYR49.5 million. Authorities allege misdeclaration during transshipment; origin, final destination, chip models and legal findings remain under investigation. Export controls and transit permits affect international GPU and server movements. Customs seizures are not a measure of legitimate server shipping volume. Reuters cited customs saying transshipment required a trade permit and that at least five suspected related cases involved more than MYR100 million in total seized chips. MYR49.5 million refers specifically to the October 15 interception. Charges, convictions, shipment origin/destination, chip specifications, customers and disposition remain undisclosed. Location: KL International Airport free trade zone, Sepang, Selangor, Malaysia (customs seizure site).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C34" s="6">
+        <v>46310</v>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and test-equipment logistics providers would distinguish declarations, origin documentation and required permits. The investigation does not establish wrongdoing by any named manufacturer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-30 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-25-en.xlsx
+++ b/docs/exports/week-2026-10-25-en.xlsx
@@ -134,22 +134,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Memory modules, materials and high-speed chips
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">ITRI presented a rare-earth plan, Tenghui's Thai CCL plant began small shipments and Macronix memory expansion targets 2027. TeamGroup plans Q2 2027 module production while Parade guided lower Q4 interface-chip revenue; actuals, plans and forecasts have different statuses.</t>
+            <t xml:space="preserve">Memory, passive components and electronics materials
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">ITRI and Tenghui disclosed rare-earth and Thai PCB-materials developments, while Macronix and TeamGroup target 2027 capacity ramps. On October 29 Yageo reported an AI mix near 20% and high MLCC/tantalum utilization, with future capacity still to be qualified.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 24, Oct 26, Oct 27, Oct 28</t>
+          <t xml:space="preserve">Oct 24, Oct 26, Oct 27, Oct 28, Oct 29</t>
         </is>
       </c>
     </row>
@@ -168,22 +168,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Wafer testing, factory automation and precision tools
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Grid restoration, Foxconn's AI manufacturing measurements and a NARLabs/MSS high-NA EUV metrology method represent separate stages. CHPT reported probe-card results and a 2027 capacity target on October 28, while Jin-An opened its Longtan factory; absolute throughput and deliveries remain distinct.</t>
+            <t xml:space="preserve">Factory automation, process metrology and industrial systems
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taipower restoration, Foxconn workflow measurements and NARLabs high-NA EUV metrology reflect different operating evidence. CHPT described probe-card capacity and Jin-An opened a thermal plant; Advantech reported Q3 revenue of NT$32.44B and book-to-bill of 1.64 across industrial and equipment demand.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26, Oct 27, Oct 28</t>
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26, Oct 27, Oct 28, Oct 29</t>
         </is>
       </c>
     </row>
@@ -202,22 +202,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Power and data-center infrastructure across Taiwan and Southeast Asia
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">MViSTA remains in tender, Malaysia's US$50B intention lacks approved projects and Singapore granted conditional power-import approval. Delta published Q3 results and Chief Telecom described data-center revenue and an LY2 occupancy goal; financial results, intentions and energized capacity are different measures.</t>
+            <t xml:space="preserve">Data-center power, server financing and Southeast Asian power components
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">MViSTA's cable tender, Malaysia's data-center investment intention and Singapore's conditional 1.3GW power approval are not commissioned facilities. On October 29 Delta described delayed sites and inventory write-downs, Gigabyte approved NT$50B credit, and Thailand-based JPP reported a power-cabinet and BBU enclosure ramp.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 26, Oct 27, Oct 28</t>
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 26, Oct 27, Oct 28, Oct 29</t>
         </is>
       </c>
     </row>
@@ -236,22 +236,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Advanced packaging, optics and electronics test equipment
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">GSEO and 3M's optical interconnect has no published customer volume qualification, while Powertech's advanced packaging share exceeds 30% but FOPLP awaits qualification. ASMPT's SMT divestiture remains unsigned and WIN reported Q3 results and a photodiode ramp on October 28, with future deliveries unconfirmed.</t>
+            <t xml:space="preserve">Advanced packaging, optics and semiconductor test tooling
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Powertech's advanced packaging mix and CHPT's probe-card results were reported this week while FOPLP and CPO remain in qualification. ASMPT's SMT sale is unsigned and WIN optical receivers are ramping. KYEC announced Texas property and around US$534M of tool purchases on October 29, with 2027 production still targeted.</t>
           </r>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 23, Oct 25, Oct 26, Oct 27, Oct 28</t>
+          <t xml:space="preserve">Oct 23, Oct 25, Oct 26, Oct 27, Oct 28, Oct 29</t>
         </is>
       </c>
     </row>
@@ -270,22 +270,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Wafer fabrication, regional cooperation and chip controls
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Philippine semiconductor corridors remain policy discussions, Reuters reported incomplete Viettel fab and DUV milestones, and Faraday disclosed a 2nm design project. UMC authorized about US$3.2B extra expansion on October 28; Malaysian customs separately disclosed an October 15 AI-server seizure, with distinct approval and enforcement dates.</t>
+            <t xml:space="preserve">Wafer facilities, chip design and sector policy
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Philippine cooperation remains policy discussion, Viettel's fab and DUV status are disputed, Faraday reported a 2nm design project and UMC approved extra expansion budget. On October 29 AUO authorized a NT$38.8B factory sale to TSMC and TSIA forecast annual output above NT$9.1T; property, design, capex and output forecasts are distinct.</t>
           </r>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 15, Oct 24, Oct 26, Oct 27, Oct 28</t>
+          <t xml:space="preserve">Oct 15, Oct 24, Oct 26, Oct 27, Oct 28, Oct 29</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="310" customHeight="1">
+    <row r="9" ht="262" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">07</t>
@@ -572,6 +572,43 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Yageo reports NT$49.532B Q3 revenue and near-20% AI mix; Q4 utilization above 95% is guidance
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At its October 29 briefing, Yageo reported Q3 revenue of NT$49.532 billion, 41% gross margin and NT$11.981 billion attributable profit. AI-related revenue mix increased from 16% in Q2 to nearly 20% in Q3; Q4 utilization above 95% and a staged 10% to 15% capacity expansion into 2027 are management targets. MLCCs, tantalum capacitors and specialty components support server power, communications and industrial systems. AI revenue mix cannot be converted into rack shipment volume or specific capacitor units. Yageo said Q3 book-to-bill was near two, both standard and specialty utilization approached 95%, and supply agreements were discussed with major customers. Q4 and 2027 figures are guidance distinct from recognized Q3 sales. AI-specific MLCC/tantalum unit output, absolute new capacity, contract pricing and tool spending remain undisclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C9" s="6">
+        <v>46324</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server power-conversion and test suppliers would verify component electrical and reliability specifications and line qualification schedules. Revenue mix and forecast utilization are not equipment purchase commitments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="310" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Taipower reports over 340,000 storm-affected accounts and more than 90% restored
 </t>
           </r>
@@ -585,22 +622,22 @@
           </r>
         </is>
       </c>
-      <c r="C9" s="6">
+      <c r="C10" s="6">
         <v>46319</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion and industrial power-quality suppliers would separate distribution failure from on-site backup behavior and review insulation protection, UPS transfer and observed voltage events. Without site-level records, tool downtime and lost output cannot be inferred.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="294" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
+    <row r="11" ht="294" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -622,22 +659,22 @@
           </r>
         </is>
       </c>
-      <c r="C10" s="6">
+      <c r="C11" s="6">
         <v>46317</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial power, machine-vision test and edge compute hardware suppliers would seek camera, server and appliance specifications and site acceptance requirements. No deployment volumes or factory customer contracts were disclosed.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="358" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">09</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+    <row r="12" ht="358" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -659,49 +696,12 @@
           </r>
         </is>
       </c>
-      <c r="C11" s="6">
+      <c r="C12" s="6">
         <v>46320</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, UPS and plant monitoring suppliers would review actual voltage dips, storage transfer events and plant alerts. Household restoration totals do not measure tool availability or backup equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="178" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn and NVIDIA report 25% lower scheduling labor hours
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn and NVIDIA reported October 26 that scheduling labor hours fell 25% and molding engineering work fell 50% in selected manufacturing processes. A specified model-training task ran 2.48 times faster on DGX than an older H100 system; cross-factory validation was not disclosed. Applications span SMT, scheduling, automation, metrology and server AI training. NVIDIA cites an H100 comparison and one trillion tokens processed over 12 days; selected workflow outcomes are not factory-wide averages. Test sites, absolute baseline hours and line yield data remain undisclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C12" s="6">
-        <v>46321</v>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Metrology and process-power suppliers would verify baseline labor hours and site scope. Results cannot be generalized without controlled samples.</t>
         </is>
       </c>
     </row>
@@ -720,16 +720,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">JIMTOF opens in Tokyo with 94 Taiwan exhibitors, association says
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">JIMTOF opened October 26 at Tokyo Big Sight, running through October 31. Taiwan's machine-tool association reported 94 participating companies covering CNC, metrology and automation; new orders were not disclosed. Precision machinery and controls support industrial automation and semiconductor tool components; exhibiting is not a signed order. Organizer confirms October 26-31 at Tokyo Big Sight; exhibitor number was reported by CNA. Signed deals, qualification and equipment procurement are unknown. Location: Tokyo Big Sight, Tokyo, Japan (exhibition venue).</t>
+            <t xml:space="preserve">Foxconn and NVIDIA report 25% lower scheduling labor hours
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn and NVIDIA reported October 26 that scheduling labor hours fell 25% and molding engineering work fell 50% in selected manufacturing processes. A specified model-training task ran 2.48 times faster on DGX than an older H100 system; cross-factory validation was not disclosed. Applications span SMT, scheduling, automation, metrology and server AI training. NVIDIA cites an H100 comparison and one trillion tokens processed over 12 days; selected workflow outcomes are not factory-wide averages. Test sites, absolute baseline hours and line yield data remain undisclosed.</t>
           </r>
         </is>
       </c>
@@ -738,17 +738,54 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Metrology and process-power suppliers would verify baseline labor hours and site scope. Results cannot be generalized without controlled samples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="178" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">JIMTOF opens in Tokyo with 94 Taiwan exhibitors, association says
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">JIMTOF opened October 26 at Tokyo Big Sight, running through October 31. Taiwan's machine-tool association reported 94 participating companies covering CNC, metrology and automation; new orders were not disclosed. Precision machinery and controls support industrial automation and semiconductor tool components; exhibiting is not a signed order. Organizer confirms October 26-31 at Tokyo Big Sight; exhibitor number was reported by CNA. Signed deals, qualification and equipment procurement are unknown. Location: Tokyo Big Sight, Tokyo, Japan (exhibition venue).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C14" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Equipment-power and precision metrology suppliers would verify tool specifications and customer acceptance; participation does not prove sales.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="262" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
+    <row r="15" ht="262" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -767,43 +804,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">NARLabs announced October 27 that its instrumentation center and Materials Analysis Technology Inc. (MSS) developed a coating approach to stabilize high-NA EUV metal-oxide-resist nanostructures for subsequent wafer cross-section analysis. NARLabs says it helped MSS enter major semiconductor suppliers' process chains, without customer acceptance, yield or deployment volumes. High-NA EUV metal-oxide-resist patterns require structural preservation during cross-section sample preparation, linking advanced lithography to metrology and microscopy. NARLabs describes stabilizing fragile patterned structures with coating prior to analysis. The disclosed research milestone is not evidence of a qualified high-volume manufacturing node. Comparative defect rates, tested resolution, fab qualification dates and commercial metrology orders were not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C14" s="6">
-        <v>46322</v>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Process-metrology, power and analysis-tool suppliers would examine material compatibility, specimen reproducibility and qualification. Research success does not establish volume tool contracts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="246" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Hongwei says specialized industrial lift orders now provide three years of visibility
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">On October 27, Hongwei Electric said its backlog for heavy-duty, cleanroom and automated material-handling lifts now offers three years of visibility, with orders on hand doubling versus 2025. It described semiconductor-related shipments as roughly 59% of the relevant mix, without disclosing absolute contract value or customer site details. Cleanroom, heavy-load and explosion-proof lifts support factory logistics and utilities, not front-end lithography or process equipment. Management said orders-to-shipments remained above one and reported sales to semiconductor and testing-related customers; three-year backlog visibility is a company estimate, not realized revenue. Absolute backlog units, contract values, delivery schedule and named project sites were not disclosed or independently verified.</t>
           </r>
         </is>
       </c>
@@ -812,7 +812,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industrial power and material-handling suppliers would seek delivery sites, load ratings and acceptance milestones. Backlog visibility is not recognized revenue or evidence of wafer-fab commissioning.</t>
+          <t xml:space="preserve">Process-metrology, power and analysis-tool suppliers would examine material compatibility, specimen reproducibility and qualification. Research success does not establish volume tool contracts.</t>
         </is>
       </c>
     </row>
@@ -831,6 +831,43 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Hongwei says specialized industrial lift orders now provide three years of visibility
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 27, Hongwei Electric said its backlog for heavy-duty, cleanroom and automated material-handling lifts now offers three years of visibility, with orders on hand doubling versus 2025. It described semiconductor-related shipments as roughly 59% of the relevant mix, without disclosing absolute contract value or customer site details. Cleanroom, heavy-load and explosion-proof lifts support factory logistics and utilities, not front-end lithography or process equipment. Management said orders-to-shipments remained above one and reported sales to semiconductor and testing-related customers; three-year backlog visibility is a company estimate, not realized revenue. Absolute backlog units, contract values, delivery schedule and named project sites were not disclosed or independently verified.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C16" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial power and material-handling suppliers would seek delivery sites, load ratings and acceptance milestones. Backlog visibility is not recognized revenue or evidence of wafer-fab commissioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="246" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Follow-up: CHPT reports nearly NT$400M Q3 advanced probe-card sales and 3x capacity target
 </t>
           </r>
@@ -841,43 +878,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">At an October 28 briefing, CHPT said advanced probe cards contributed nearly NT$400 million or 21% of Q3 revenue, while HPC products represented 65.9%. Capacity had doubled relative to end-2025 by August, with a threefold level targeted for Q1 2027, adding operational detail to the previous day's earnings. Probe cards, wafer test boards and high-power burn-in systems serve GPUs, TPUs, ASICs and CPO testing. Signal, power-integrity and temperature requirements differ by product. Management expects engineering CPU probe-card samples in November and targets volume production in 2027; CPO test interface talks involve more than five firms. These are stated qualification and commercial milestones, not completed acceptance. Absolute throughput, channel counts, accepted customers and high-power burn-in board volumes remain undisclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C16" s="6">
-        <v>46323</v>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Test-power, prober and burn-in suppliers would verify power density, channel requirements and qualification dates. A capacity multiple without absolute unit throughput cannot determine equipment volumes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="310" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Jin-An Machinery opens Longtan plant for ice-storage cooling and industrial unmanned systems
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">I-Mei affiliate Jin-An Machinery opened a new manufacturing building in Longtan, Taoyuan on October 28, following investment above NT$1 billion. The facility plans to make more than 20 off-peak ice-storage cooling systems for group factories; management claims a 25% to 30% reduction in peak electricity draw at an existing Longtan site, not a universal efficiency result. Ice-storage cooling shifts HVAC electricity loads from daytime to off-peak hours, rather than directly reducing chip-cooling load or total kWh. Unmanned systems and environmental tests are a separate line of work. The facility houses freeze-drying, thermal-storage and unmanned-system production. The above-NT$1B figure is a company-stated project total without tool/facility breakdown; 20-plus cooling systems are prospective production. Construction periods, individual system kW ratings, measured kWh and external customer acceptance counts are unavailable. Location: Longtan District, Taoyuan City, Taiwan, Jin-An manufacturing building (opened site, street address not verified).</t>
           </r>
         </is>
       </c>
@@ -886,17 +886,91 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Test-power, prober and burn-in suppliers would verify power density, channel requirements and qualification dates. A capacity multiple without absolute unit throughput cannot determine equipment volumes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="310" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Jin-An Machinery opens Longtan plant for ice-storage cooling and industrial unmanned systems
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">I-Mei affiliate Jin-An Machinery opened a new manufacturing building in Longtan, Taoyuan on October 28, following investment above NT$1 billion. The facility plans to make more than 20 off-peak ice-storage cooling systems for group factories; management claims a 25% to 30% reduction in peak electricity draw at an existing Longtan site, not a universal efficiency result. Ice-storage cooling shifts HVAC electricity loads from daytime to off-peak hours, rather than directly reducing chip-cooling load or total kWh. Unmanned systems and environmental tests are a separate line of work. The facility houses freeze-drying, thermal-storage and unmanned-system production. The above-NT$1B figure is a company-stated project total without tool/facility breakdown; 20-plus cooling systems are prospective production. Construction periods, individual system kW ratings, measured kWh and external customer acceptance counts are unavailable. Location: Longtan District, Taoyuan City, Taiwan, Jin-An manufacturing building (opened site, street address not verified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C18" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Industrial cooling, drives and power-controls suppliers would verify thermal-storage size, load profiles and peak demand calculations. A single site's reduction is not a universal data-center efficiency result.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="400" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
+    <row r="19" ht="246" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Advantech reports NT$32.44B Q3 revenue and NT$6.218B profit amid industrial demand
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Advantech released Q3 results on October 29: NT$32.44 billion revenue, up 83% YoY, and NT$6.218 billion net income, up 125%, with EPS of NT$7.15. The company cited semiconductor equipment, edge AI and healthcare demand and a Q3 book-to-bill ratio of 1.64, which is not a revenue growth rate. Industrial computers and embedded edge systems serve factory automation, semiconductor tools and medical devices. Regional book-to-bill uses order and shipment values rather than capacity utilization. Advantech's primary release shows 24% QoQ revenue growth, NT$6.795B operating profit and NT$6.218B net income. CNA cites management on regional book-to-bill ratios of 2.12 for North America, 1.52 for Europe and 1.50 for China. Product-specific revenue, equipment installations and customer delivery schedules by application were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C19" s="6">
+        <v>46324</v>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial metrology, precision power and semiconductor-tool suppliers would distinguish applications and geography and verify deliveries. Book-to-bill indicates order flow, not the specific downstream deployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="400" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -918,22 +992,22 @@
           </r>
         </is>
       </c>
-      <c r="C18" s="6">
+      <c r="C20" s="6">
         <v>46317</v>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power, liquid-cooling and metrology suppliers would track the cable tender separately from Vietnam campus feasibility and site power agreements. Landing stations, anchor tenants, power contracts and construction permits are still missing.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="400" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
+    <row r="21" ht="400" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -955,22 +1029,22 @@
           </r>
         </is>
       </c>
-      <c r="C19" s="6">
+      <c r="C21" s="6">
         <v>46319</v>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion, UPS, power-quality and liquid-cooling suppliers would verify specific sites, permitted MW load, qualification and purchasing milestones. An aggregate intention without allocation cannot indicate equipment deliveries.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="214" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
+    <row r="22" ht="214" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -992,22 +1066,22 @@
           </r>
         </is>
       </c>
-      <c r="C20" s="6">
+      <c r="C22" s="6">
         <v>46321</v>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power conversion and data-center suppliers need transmission specifications, storage designs and offtake terms. No finalized construction or financing plans are available.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="278" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
+    <row r="23" ht="278" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1029,22 +1103,22 @@
           </r>
         </is>
       </c>
-      <c r="C21" s="6">
+      <c r="C23" s="6">
         <v>46322</v>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Smart-factory power and test suppliers would check equipment type, whether transferred or newly built, and acceptance status. An intercompany book transaction cannot establish incremental production capacity.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="230" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+    <row r="24" ht="230" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1066,22 +1140,22 @@
           </r>
         </is>
       </c>
-      <c r="C22" s="6">
+      <c r="C24" s="6">
         <v>46323</v>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power and industrial metrology suppliers would separate group results from actual delivery of data-center modules and monitor later product qualification disclosures. Consolidated sales alone cannot quantify new rack deployment.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="262" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">21</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
+    <row r="25" ht="262" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1103,90 +1177,16 @@
           </r>
         </is>
       </c>
-      <c r="C23" s="6">
+      <c r="C25" s="6">
         <v>46323</v>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">UPS, power and liquid-cooling suppliers would verify the occupancy denominator, energized racks and power per cabinet. An 80% tenancy goal is not an equipment purchase count.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="342" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C24" s="6">
-        <v>46318</v>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="374" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">EVA Air cites sustained high-tech airfreight demand; September cargo revenue rose 42.55%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Speaking in Taipei on October 25, EVA Air president Clay Sun said AI server and other high-tech airfreight demand remained strong through the year, supporting cargo rates, while aviation fuel costs pressured margins. Previously released September cargo revenue was NT$6.167 billion, up 42.55% year on year; it is historical monthly revenue, not October 25 shipment volume. Air cargo transports Taiwan-origin AI servers, racks, semiconductor equipment and high-value electronics. Different cargo types impose distinct weight, space, handling and time constraints; freight revenue cannot be translated directly into equipment production capacity. Management said on October 25 that aviation fuel had reached approximately US$177 per barrel at one point, and that fares and freight rates had been adjusted. September consolidated revenue of NT$20.749 billion and cargo revenue of NT$6.167 billion are earlier reported results, not exclusively AI-related revenue. Cargo-revenue growth reflects shipment volume, rates and product mix, but the report gives no decomposition. US$177 a barrel is a past fuel price referenced by an executive, not a verified spot quote for October 25. Same-day cargo load factors, AI-specific tonnage, long-term customer contracts, fuel-hedging coverage and incremental dedicated freight contracts were not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C25" s="6">
-        <v>46320</v>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="230" customHeight="1">
+    <row r="26" ht="262" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">24</t>
@@ -1201,25 +1201,25 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Reuters: Bidding on ASMPT's SMT business continues with no signed sale
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Reuters reported October 26 that IDG Capital was the leading bidder for Singapore-headquartered ASMPT's SMT business, with a potential deal value above US$1 billion, but no agreement finalized. ASMPT's January strategic review considered sale, joint venture, spin-off, listing or retention. SMT equipment covers board printing, placement and inspection for servers, transceivers and electronics. Reported bidding does not establish service or warranty changes. Reuters cited H1 SMT revenue growth of 53.1% to HK$3.87 billion and bookings growth of 87.8% to HK$6.98 billion. Those are historical results; bidder progress is the new claim. No signed agreement, final buyer, price, regulatory filings or workforce plan confirmed.</t>
+            <t xml:space="preserve">Follow-up: Delta attributes Q3 inventory write-down to data-center delays and supply mismatches
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At an October 29 investor briefing, Delta chairman Ping Cheng said delayed data-center projects and shortages/excesses in component supply contributed to inventory write-downs equal to about 1.7% of Q3 revenue. Management expects Q4 sales to exceed Q3, while power infrastructure, labor, materials and local permitting remain schedule constraints. Data-center HVDC, UPS, substations and cooling systems depend on site construction and grid readiness. Supplier inventory is not proof of end-customer rack deployment. The previous day's reported Q3 attributable profit of NT$23.495 billion is historical context. New October 29 comments describe inventory write-downs and project execution constraints; 1.7% of revenue is not equipment failure incidence. Project delay days by site, affected customers, actual Q4 inventory reversal and product-specific order volumes remain undisclosed.</t>
           </r>
         </is>
       </c>
       <c r="C26" s="6">
-        <v>46321</v>
+        <v>46324</v>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMT power, test and service suppliers would track any formal ownership and warranty changes. Reported bidding does not establish a contract transfer.</t>
+          <t xml:space="preserve">Data-center power and measurement suppliers would verify customers' grid readiness, electricians and equipment acceptance milestones. Inventory impairments reflect schedule and supply-mix issues, not necessarily product defects.</t>
         </is>
       </c>
     </row>
@@ -1238,29 +1238,29 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Powertech says advanced packaging exceeds 30% of revenue and utilization tops 90%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Powertech Technology reported October 27 third-quarter revenue of NT$25.334 billion, 24% gross margin and NT$2.612 billion in profit attributable to shareholders. It said advanced packaging now exceeds 30% of group revenue and packaging/test utilization topped 90% in Q3; FOPLP qualification, the 2027 production target and its Singapore investment remain pending. The company serves DRAM, NAND/eSSD and logic packaging, with planned FOPLP, FCBGA, heterogeneous integration and optical engines for CPO. These product types cannot be counted as one commissioned capacity. Large-die FCBGA entered production in Q3 according to management, with larger packages slated for Q4. FOPLP remains a 2027 target, and potential alliances with foundries are not signed agreements. FOPLP customer acceptance, absolute monthly capacity, Singapore investment size and shipment dates were not disclosed.</t>
+            <t xml:space="preserve">Gigabyte board approves NT$50B syndicated credit for debt refinancing and AI working capital
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 29, Gigabyte's board approved a NT$50 billion syndicated credit facility led by Bank of Taiwan, Mega Bank, Hua Nan and Cathay United Bank. The facility is intended for refinancing and medium-term working capital, including preparation for 2027 AI products; committed credit is not drawn cash, new sales or customer orders. Gigabyte makes motherboards, GPUs, AI servers and systems, using working capital for chip, memory and assembly procurement. Bank credit approval does not prove component shipments or production of particular systems. The banking syndicate includes Bank of Taiwan, Mega, Hua Nan and Cathay United. Gigabyte did not provide the allocation between refinancing and AI procurement, nor amounts actually drawn. Drawdown, actual component purchases, customer shipments, financing costs and timing of inventory build remain undisclosed.</t>
           </r>
         </is>
       </c>
       <c r="C27" s="6">
-        <v>46322</v>
+        <v>46324</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Packaging tool, test-power and metrology suppliers would check qualified package sizes, line requirements and actual delivery milestones. Q3 utilization and future expansion are separate measures, not equipment orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="230" customHeight="1">
+          <t xml:space="preserve">Server power, rack distribution and electronic test suppliers would verify actual procurement schedules and customer acceptance. Credit capacity cannot be translated into rack volumes or module purchase orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="326" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">26</t>
@@ -1275,29 +1275,29 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">CHPT reports NT$1.905B Q3 sales and NT$551M profit; probe cards lead mix
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">CHPT's board approved October 27 Q3 results showing NT$1.905 billion revenue, up 53.4% YoY, and NT$551 million attributable profit, up 100% YoY. Wafer probe cards accounted for 71% of Jan-Sep revenue and IC load boards for 21%; next-generation customer qualification data is not public. Wafer probe cards and IC load boards support wafer sorting and package test for memory and AI ASICs. Revenue mix is not production quantity. Its primary release reports 57.3% Q3 gross margin and roughly 35% operating margin, citing demand for customized AI testing interfaces. It gives growth rates without every absolute prior-year base. Next-generation probe-card customer roster, utilization, qualification times and new tool investments were not disclosed.</t>
+            <t xml:space="preserve">Thailand-based JPP reports power-cabinet and BBU component production ramp in Q4
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 29, Taiwan-listed JPP, which manufactures in Thailand, said it had entered a Thai power-management supplier's chain and targets Q4 volume production of power cabinets, battery backup unit (BBU) housings and server components. It separately reported 20 Airbus A350 aerospace process qualifications, while actual electrical-product shipment volumes and acceptance remain undisclosed. Precision sheet-metal enclosures support rack power distribution, BBU systems and server chassis but are distinct from converters and battery cells. Aerospace qualifications concern another product category, not electrical system validation. Management described a partnership with a Thai power-management company and a Q4 production ramp, without named product SKUs, lines or customer delivery orders. The 20 aerospace certifications do not quantify BBU production. Monthly power-cabinet and BBU shipments, electrical test standards, customer sign-off and North American data-center delivery timing are unknown. Location: JPP manufacturing operations in Thailand (site referenced by company; specific factory address not disclosed).</t>
           </r>
         </is>
       </c>
       <c r="C28" s="6">
-        <v>46322</v>
+        <v>46324</v>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">High-frequency test-power and probe-card suppliers would seek channel-level signal/power-integrity specifications and qualification timelines. Sales mix cannot quantify tester procurement or throughput.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="246" customHeight="1">
+          <t xml:space="preserve">Rack-power, BBU and industrial-power suppliers would verify mechanical thermal, insulation, EMI and reliability qualifications. Production plans without order volumes do not establish deployed data-center power.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="342" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">27</t>
@@ -1312,29 +1312,29 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">WIN Semiconductors Q3 sales reach NT$5.859B; photodiode ramp ongoing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">WIN Semiconductors announced October 28 Q3 revenue of NT$5.859 billion, gross margin 37.4% and attributable profit of NT$1.93 billion. Optical receiver photodiodes remain in early production ramp, with management pointing to larger-scale shipments in 2028; application-level volume was not reported. WIN's GaAs RF and receiver products serve satellite links, optical communications and data-center modules. Revenue growth is not evidence of new wafer-fab commissioning. Management said gross margin rose 9.2 percentage points from Q2 and profit increased around 98% sequentially. Q4 revenue guidance is low-single-digit sequential growth amid mixed handset demand. PD monthly shipments, yields, qualified customers and planned 2028 capacity allocations were not disclosed.</t>
+            <t xml:space="preserve">GSEO reports NT$434M September net profit as 3M placement proceeds arrive
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Genius Electronic Optical reported October 23 self-compiled September profit attributable to owners of about NT$434 million, down 15% year on year, and EPS of NT$3.85. Separate reporting said 3M's roughly NT$4.813 billion private-placement payment had arrived. Earlier cooperation covers Expanded Beam Optical, co-packaged optics and data-center interconnects, without a confirmed customer production ramp. GSEO's precision optics production is intended to support 3M's EBO ferrules and optical interconnect development. This links precision optical materials, advanced packaging and data-center networking, while September financial performance cannot be attributed to products not yet in volume production. 3M's October 19 release said it expected to acquire approximately 4.7% of GSEO subject to customary closing conditions, while October 23 reporting said funds were remitted. CNA reported Q3 revenue around NT$7.812 billion, up about 1%, and parent-attributable net profit around NT$1.092 billion, down about 23%, which are separate quarterly figures. Final legal closing, EBO manufacturing yields, customer qualification and shipment schedules remain undisclosed; reported profits are self-compiled.</t>
           </r>
         </is>
       </c>
       <c r="C29" s="6">
-        <v>46323</v>
+        <v>46318</v>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">RF process-power and optical metrology suppliers would verify PD yields and receiver test bandwidth. Future volume projections cannot be inferred from consolidated profit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="342" customHeight="1">
+          <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="374" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">28</t>
@@ -1349,29 +1349,29 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
+            <t xml:space="preserve">EVA Air cites sustained high-tech airfreight demand; September cargo revenue rose 42.55%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Speaking in Taipei on October 25, EVA Air president Clay Sun said AI server and other high-tech airfreight demand remained strong through the year, supporting cargo rates, while aviation fuel costs pressured margins. Previously released September cargo revenue was NT$6.167 billion, up 42.55% year on year; it is historical monthly revenue, not October 25 shipment volume. Air cargo transports Taiwan-origin AI servers, racks, semiconductor equipment and high-value electronics. Different cargo types impose distinct weight, space, handling and time constraints; freight revenue cannot be translated directly into equipment production capacity. Management said on October 25 that aviation fuel had reached approximately US$177 per barrel at one point, and that fares and freight rates had been adjusted. September consolidated revenue of NT$20.749 billion and cargo revenue of NT$6.167 billion are earlier reported results, not exclusively AI-related revenue. Cargo-revenue growth reflects shipment volume, rates and product mix, but the report gives no decomposition. US$177 a barrel is a past fuel price referenced by an executive, not a verified spot quote for October 25. Same-day cargo load factors, AI-specific tonnage, long-term customer contracts, fuel-hedging coverage and incremental dedicated freight contracts were not disclosed.</t>
           </r>
         </is>
       </c>
       <c r="C30" s="6">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="294" customHeight="1">
+          <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="230" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">29</t>
@@ -1386,16 +1386,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Reuters: Viettel fab lacks buildings and DUV equipment deal remains pending
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Reuters reported October 26 that no buildings have been constructed at Viettel's planned wafer fab outside Hanoi since a January groundbreaking and talks to purchase a DUV lithography tool from ASML remain unresolved. Sources doubt the 2027 trial-production target, whereas Viettel says progress remains in line with its plan. Vietnam already hosts Intel, Amkor and Hana Micron packaging/test sites. Viettel's proposed front-end fab would require lithography, deposition, etch, process power and utilities, distinct from installed packaging capacity. Reuters' site visit and satellite images found no buildings. Authorities previously estimated US$1.3 billion cost, a 2027 trial and full operation by 2030. Viettel says phased progress continues, while ASML has not confirmed a contract. DUV tool type, a signed procurement contract, construction permits, technology partner and validated trial date remain unknown. Location: Planned Viettel wafer fab site on the outskirts of Hanoi, Vietnam (industrial estate not specified).</t>
+            <t xml:space="preserve">Reuters: Bidding on ASMPT's SMT business continues with no signed sale
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Reuters reported October 26 that IDG Capital was the leading bidder for Singapore-headquartered ASMPT's SMT business, with a potential deal value above US$1 billion, but no agreement finalized. ASMPT's January strategic review considered sale, joint venture, spin-off, listing or retention. SMT equipment covers board printing, placement and inspection for servers, transceivers and electronics. Reported bidding does not establish service or warranty changes. Reuters cited H1 SMT revenue growth of 53.1% to HK$3.87 billion and bookings growth of 87.8% to HK$6.98 billion. Those are historical results; bidder progress is the new claim. No signed agreement, final buyer, price, regulatory filings or workforce plan confirmed.</t>
           </r>
         </is>
       </c>
@@ -1404,11 +1404,11 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wafer process-power and metrology suppliers would check signed equipment orders, process partnerships and building permits. Differing site evidence and developer statements leave the 2027 milestone unconfirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="246" customHeight="1">
+          <t xml:space="preserve">SMT power, test and service suppliers would track any formal ownership and warranty changes. Reported bidding does not establish a contract transfer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="262" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">30</t>
@@ -1423,16 +1423,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Faraday secures Samsung 2nm GAA design project, targets first revenue in H1 2027
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">On October 27, Faraday Technology announced a U.S. cloud AI chip non-recurring engineering project using Samsung's 2nm GAA foundry, with UMC and memory partners. Management described project value in the tens of millions of U.S. dollars and expects initial revenue recognition in H1 2027, without a precise contract value or qualified production date. The design project requires advanced-node IP and coordination across foundry and memory partners. UMC's participation does not make it the 2nm wafer foundry. Q3 revenue was NT$3.664B, gross margin 42.5% and attributable profit NT$279M. Management attributed margin changes partly to product mix and profit changes partly to non-operating valuation gains. Customer identity, package technology, exact NRE timing and chip shipment volumes were not given.</t>
+            <t xml:space="preserve">Powertech says advanced packaging exceeds 30% of revenue and utilization tops 90%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Powertech Technology reported October 27 third-quarter revenue of NT$25.334 billion, 24% gross margin and NT$2.612 billion in profit attributable to shareholders. It said advanced packaging now exceeds 30% of group revenue and packaging/test utilization topped 90% in Q3; FOPLP qualification, the 2027 production target and its Singapore investment remain pending. The company serves DRAM, NAND/eSSD and logic packaging, with planned FOPLP, FCBGA, heterogeneous integration and optical engines for CPO. These product types cannot be counted as one commissioned capacity. Large-die FCBGA entered production in Q3 according to management, with larger packages slated for Q4. FOPLP remains a 2027 target, and potential alliances with foundries are not signed agreements. FOPLP customer acceptance, absolute monthly capacity, Singapore investment size and shipment dates were not disclosed.</t>
           </r>
         </is>
       </c>
@@ -1441,17 +1441,239 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Packaging tool, test-power and metrology suppliers would check qualified package sizes, line requirements and actual delivery milestones. Q3 utilization and future expansion are separate measures, not equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="230" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">CHPT reports NT$1.905B Q3 sales and NT$551M profit; probe cards lead mix
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">CHPT's board approved October 27 Q3 results showing NT$1.905 billion revenue, up 53.4% YoY, and NT$551 million attributable profit, up 100% YoY. Wafer probe cards accounted for 71% of Jan-Sep revenue and IC load boards for 21%; next-generation customer qualification data is not public. Wafer probe cards and IC load boards support wafer sorting and package test for memory and AI ASICs. Revenue mix is not production quantity. Its primary release reports 57.3% Q3 gross margin and roughly 35% operating margin, citing demand for customized AI testing interfaces. It gives growth rates without every absolute prior-year base. Next-generation probe-card customer roster, utilization, qualification times and new tool investments were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C33" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-frequency test-power and probe-card suppliers would seek channel-level signal/power-integrity specifications and qualification timelines. Sales mix cannot quantify tester procurement or throughput.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="246" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">WIN Semiconductors Q3 sales reach NT$5.859B; photodiode ramp ongoing
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">WIN Semiconductors announced October 28 Q3 revenue of NT$5.859 billion, gross margin 37.4% and attributable profit of NT$1.93 billion. Optical receiver photodiodes remain in early production ramp, with management pointing to larger-scale shipments in 2028; application-level volume was not reported. WIN's GaAs RF and receiver products serve satellite links, optical communications and data-center modules. Revenue growth is not evidence of new wafer-fab commissioning. Management said gross margin rose 9.2 percentage points from Q2 and profit increased around 98% sequentially. Q4 revenue guidance is low-single-digit sequential growth amid mixed handset demand. PD monthly shipments, yields, qualified customers and planned 2028 capacity allocations were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C34" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RF process-power and optical metrology suppliers would verify PD yields and receiver test bandwidth. Future volume projections cannot be inferred from consolidated profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="326" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Follow-up: KYEC acquires Texas facility for US$79.35M and reports US$534M of tool purchases
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 29, Taiwan's KYEC said its U.S. subsidiary AeternZ acquired a Texas site and building for US$79.35 million and disclosed about US$534 million in equipment and fab-utility purchases from Hon.Precision, EO Technics, KLA and TRANTEK. NVIDIA's previously announced US$1.1 billion capacity prepayment is background, while an April 2027 high-volume start remains a target. KYEC serves AI GPUs and ASICs through semiconductor testing, involving handlers, test-power systems, thermal management and facility utilities. A U.S. test site expands the geographic footprint of a Taiwan supplier, but the latest milestones are real-estate and equipment procurement. KYEC disclosed about 1,179,700 square feet of land and 489,494 square feet of buildings. Real-estate and tool transactions total roughly US$613 million as separate disclosed purchases; NVIDIA's US$1.1B prepayment is not an additional project cost to add to those figures. Exact Texas address, equipment acceptance dates, monthly test throughput, yields and first customer acceptance remain undisclosed. Location: AeternZ semiconductor test site in Texas, United States (land/building acquired; street address undisclosed).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C35" s="6">
+        <v>46324</v>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Semiconductor test-power, precision metrology and thermal suppliers would verify purchased tool configuration, site bring-up and customer acceptance requirements. Procurement disclosures do not establish qualified 2027 output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="342" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C36" s="6">
+        <v>46319</v>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="294" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Reuters: Viettel fab lacks buildings and DUV equipment deal remains pending
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Reuters reported October 26 that no buildings have been constructed at Viettel's planned wafer fab outside Hanoi since a January groundbreaking and talks to purchase a DUV lithography tool from ASML remain unresolved. Sources doubt the 2027 trial-production target, whereas Viettel says progress remains in line with its plan. Vietnam already hosts Intel, Amkor and Hana Micron packaging/test sites. Viettel's proposed front-end fab would require lithography, deposition, etch, process power and utilities, distinct from installed packaging capacity. Reuters' site visit and satellite images found no buildings. Authorities previously estimated US$1.3 billion cost, a 2027 trial and full operation by 2030. Viettel says phased progress continues, while ASML has not confirmed a contract. DUV tool type, a signed procurement contract, construction permits, technology partner and validated trial date remain unknown. Location: Planned Viettel wafer fab site on the outskirts of Hanoi, Vietnam (industrial estate not specified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C37" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wafer process-power and metrology suppliers would check signed equipment orders, process partnerships and building permits. Differing site evidence and developer statements leave the 2027 milestone unconfirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="246" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Faraday secures Samsung 2nm GAA design project, targets first revenue in H1 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 27, Faraday Technology announced a U.S. cloud AI chip non-recurring engineering project using Samsung's 2nm GAA foundry, with UMC and memory partners. Management described project value in the tens of millions of U.S. dollars and expects initial revenue recognition in H1 2027, without a precise contract value or qualified production date. The design project requires advanced-node IP and coordination across foundry and memory partners. UMC's participation does not make it the 2nm wafer foundry. Q3 revenue was NT$3.664B, gross margin 42.5% and attributable profit NT$279M. Management attributed margin changes partly to product mix and profit changes partly to non-operating valuation gains. Customer identity, package technology, exact NRE timing and chip shipment volumes were not given.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C38" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Wafer process-power and advanced packaging test suppliers would verify actual foundry, package interface and qualification milestones. NRE contract value is not wafer manufacturing or equipment spending.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="310" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
+    <row r="39" ht="310" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1473,22 +1695,22 @@
           </r>
         </is>
       </c>
-      <c r="C33" s="6">
+      <c r="C39" s="6">
         <v>46323</v>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, metrology and packaging tool suppliers would verify equipment specifications and procurement schedules separately for Singapore and Tainan. Authorization and current utilization do not establish tool delivery.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="278" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
+    <row r="40" ht="278" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1510,12 +1732,86 @@
           </r>
         </is>
       </c>
-      <c r="C34" s="6">
+      <c r="C40" s="6">
         <v>46310</v>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Server and test-equipment logistics providers would distinguish declarations, origin documentation and required permits. The investigation does not establish wrongdoing by any named manufacturer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="342" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">AUO approves NT$38.8B Taichung facility sale to TSMC and cancels a separate deal
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 29, AUO's board approved selling its Taichung phase-two factory, cleanrooms and auxiliary facilities to TSMC for NT$38.8 billion, encompassing approximately 429,030 square meters of titled floor area. AUO also canceled an earlier Hwa Ya facility deal with Quanta and approved NT$5.728 billion of additional capex; the Taichung factory remains operational and transfer procedures may extend into 2027. A sale of an existing factory and cleanroom facilities relates to foundry expansion and potential packaging infrastructure. AUO separately studies glass-core substrates, redistribution layers and optical interconnects; the sold space is not evidence of commissioned semiconductor production. The property is in Anlin Section, Xitun District, Taichung. The board-approved price excludes tax, and AUO will continue using the site temporarily. Hwa Ya negotiations ended over specifications and handover timing; AUO's additional capex authorization is separate from sale proceeds. Closing date, TSMC facility conversion purpose, tool orders, wafer starts and commissioning dates have not been disclosed. Location: AUO Taichung phase-two factory, Anlin Section, Xitun District, Taichung, Taiwan (sale property, still in operation).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C41" s="6">
+        <v>46324</v>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-power, test and fab-utility suppliers would verify closing, electrical capacity and qualification of any retrofitted cleanrooms. A real-estate purchase price does not identify tool orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="326" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">TSIA forecasts Taiwan 2026 chip industry output above NT$9.1T, up 40.9%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At an October 29 annual meeting in Hsinchu, Taiwan Semiconductor Industry Association chair Hou Yong-ching projected 2026 Taiwan IC industry output above NT$9.1 trillion, roughly 40.9% higher year on year. The association also discussed electricity reliability, materials, talent and international collaboration; the full-year figure is a forecast, not audited annual output. The industry output estimate spans chip design, foundry and packaging/test activities and cannot be compared directly with a company's sales or wafer counts. The cited 2025 industry output of roughly NT$6.5 trillion is historical context. At its 30th anniversary event TSIA reported about 220 members and 12 committees, including a materials committee. Its conditional statement on reviewing nuclear energy options represents an industry association position, not a government policy decision. Verified full-year realized output, component breakdowns and the exact unrounded base underlying the 40.9% growth forecast remain unavailable. Location: Ambassador Hotel Hsinchu, Hsinchu City, Taiwan (reported event venue for TSIA's 30th anniversary).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C42" s="6">
+        <v>46324</v>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-power and metrology businesses would examine subsector output, tool capex and electricity demand separately. An aggregate industry forecast does not quantify any individual equipment category.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-31 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-25-en.xlsx
+++ b/docs/exports/week-2026-10-25-en.xlsx
@@ -134,26 +134,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Memory, passive components and electronics materials
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">ITRI and Tenghui disclosed rare-earth and Thai PCB-materials developments, while Macronix and TeamGroup target 2027 capacity ramps. On October 29 Yageo reported an AI mix near 20% and high MLCC/tantalum utilization, with future capacity still to be qualified.</t>
+            <t xml:space="preserve">Materials, PCB and dense-board expansion
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">The week covered Thai electronics materials and memory expansion plans, while Compeq on October 30 described annual capex above NT$20B from 2026 to 2028 for mSAP/HDI capacity in Taiwan, Thailand and elsewhere. Existing shipments and planned capacity are separate.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 24, Oct 26, Oct 27, Oct 28, Oct 29</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="114" customHeight="1">
+          <t xml:space="preserve">Oct 24, Oct 26, Oct 27, Oct 28, Oct 29, Oct 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">02</t>
@@ -168,26 +168,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Factory automation, process metrology and industrial systems
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taipower restoration, Foxconn workflow measurements and NARLabs high-NA EUV metrology reflect different operating evidence. CHPT described probe-card capacity and Jin-An opened a thermal plant; Advantech reported Q3 revenue of NT$32.44B and book-to-bill of 1.64 across industrial and equipment demand.</t>
+            <t xml:space="preserve">Semiconductor process, fab power and optical testing
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Factory automation and probe-card expansion were reported alongside TSMC's October 30 pump retrofit validation, reducing a specific 10 hp rating to 4 hp. Taiwan also proposed silicon-photonics testing with 2027 overseas recognition; neither is system-wide commissioning.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26, Oct 27, Oct 28, Oct 29</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="134" customHeight="1">
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 25, Oct 26, Oct 27, Oct 28, Oct 29, Oct 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="114" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -202,26 +202,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Data-center power, server financing and Southeast Asian power components
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">MViSTA's cable tender, Malaysia's data-center investment intention and Singapore's conditional 1.3GW power approval are not commissioned facilities. On October 29 Delta described delayed sites and inventory write-downs, Gigabyte approved NT$50B credit, and Thailand-based JPP reported a power-cabinet and BBU enclosure ramp.</t>
+            <t xml:space="preserve">Server power, rack capacity and cross-border supply
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Singapore's conditional imports, Delta's data-center delays and Gigabyte's financing had different statuses. Lite-On raised its power capex budget and Foxconn described doubled AI rack capacity and manufacturing roles across Taiwan, Vietnam and North America on October 30; output must be separated from shipments.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 22, Oct 24, Oct 26, Oct 27, Oct 28, Oct 29</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="114" customHeight="1">
+          <t xml:space="preserve">Oct 22, Oct 24, Oct 26, Oct 27, Oct 28, Oct 29, Oct 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">04</t>
@@ -236,26 +236,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Advanced packaging, optics and semiconductor test tooling
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Powertech's advanced packaging mix and CHPT's probe-card results were reported this week while FOPLP and CPO remain in qualification. ASMPT's SMT sale is unsigned and WIN optical receivers are ramping. KYEC announced Texas property and around US$534M of tool purchases on October 29, with 2027 production still targeted.</t>
+            <t xml:space="preserve">Advanced packaging, ASIC and semiconductor test
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Powertech and CHPT reported packaging/test results and KYEC procured Texas test tooling. MediaTek on October 30 described initial ASIC shipments and forward revenue forecasts, while ASE Q3 coverage retains source qualifications.</t>
           </r>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 23, Oct 25, Oct 26, Oct 27, Oct 28, Oct 29</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="114" customHeight="1">
+          <t xml:space="preserve">Oct 23, Oct 25, Oct 26, Oct 27, Oct 28, Oct 29, Oct 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="98" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">05</t>
@@ -270,22 +270,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Wafer facilities, chip design and sector policy
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Philippine cooperation remains policy discussion, Viettel's fab and DUV status are disputed, Faraday reported a 2nm design project and UMC approved extra expansion budget. On October 29 AUO authorized a NT$38.8B factory sale to TSMC and TSIA forecast annual output above NT$9.1T; property, design, capex and output forecasts are distinct.</t>
+            <t xml:space="preserve">Fab assets, factory investment and policy
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan fab property transactions and UMC's capex authorization have distinct timelines, while King Slide on October 30 approved NT$19.712B for two Kaohsiung slide-rail plants. Authorizations, construction contracts and commissioning are separate milestones.</t>
           </r>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 15, Oct 24, Oct 26, Oct 27, Oct 28, Oct 29</t>
+          <t xml:space="preserve">Oct 15, Oct 24, Oct 26, Oct 27, Oct 28, Oct 29, Oct 30</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="310" customHeight="1">
+    <row r="10" ht="194" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">08</t>
@@ -609,6 +609,43 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Compeq plans annual capex above NT$20B from 2026 to 2028
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 30 Compeq described planned annual capex above NT$20B in each year from 2026 to 2028 for Taiwan, China and Thailand facilities. Q3 revenue was NT$22.585B and high-layer HDI production is reported, while 2027 mSAP and satellite sales targets of NT$25B each remain forecasts. Substrates; PCB; components; servers; data centers; investment. Management says high-layer HDI boards are already produced and it plans mSAP, optical-module and satellite PCB capacity. The two NT$25B 2027 category sales expectations remain forecasts without plant-level ramp details. Three-year capex and 2027 product revenue are plans, without plant-level tool deliveries or accepted production yields.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C10" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCB process-power and test suppliers would verify mSAP/HDI tools, yields and customer qualification. Multiyear capex and sales targets lack plant-specific procurement details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="310" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Taipower reports over 340,000 storm-affected accounts and more than 90% restored
 </t>
           </r>
@@ -622,22 +659,22 @@
           </r>
         </is>
       </c>
-      <c r="C10" s="6">
+      <c r="C11" s="6">
         <v>46319</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion and industrial power-quality suppliers would separate distribution failure from on-site backup behavior and review insulation protection, UPS transfer and observed voltage events. Without site-level records, tool downtime and lost output cannot be inferred.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="294" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">09</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
+    <row r="12" ht="294" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -659,22 +696,22 @@
           </r>
         </is>
       </c>
-      <c r="C11" s="6">
+      <c r="C12" s="6">
         <v>46317</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial power, machine-vision test and edge compute hardware suppliers would seek camera, server and appliance specifications and site acceptance requirements. No deployment volumes or factory customer contracts were disclosed.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="358" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+    <row r="13" ht="358" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -696,49 +733,12 @@
           </r>
         </is>
       </c>
-      <c r="C12" s="6">
+      <c r="C13" s="6">
         <v>46320</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, UPS and plant monitoring suppliers would review actual voltage dips, storage transfer events and plant alerts. Household restoration totals do not measure tool availability or backup equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="178" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn and NVIDIA report 25% lower scheduling labor hours
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn and NVIDIA reported October 26 that scheduling labor hours fell 25% and molding engineering work fell 50% in selected manufacturing processes. A specified model-training task ran 2.48 times faster on DGX than an older H100 system; cross-factory validation was not disclosed. Applications span SMT, scheduling, automation, metrology and server AI training. NVIDIA cites an H100 comparison and one trillion tokens processed over 12 days; selected workflow outcomes are not factory-wide averages. Test sites, absolute baseline hours and line yield data remain undisclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C13" s="6">
-        <v>46321</v>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Metrology and process-power suppliers would verify baseline labor hours and site scope. Results cannot be generalized without controlled samples.</t>
         </is>
       </c>
     </row>
@@ -757,16 +757,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">JIMTOF opens in Tokyo with 94 Taiwan exhibitors, association says
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">JIMTOF opened October 26 at Tokyo Big Sight, running through October 31. Taiwan's machine-tool association reported 94 participating companies covering CNC, metrology and automation; new orders were not disclosed. Precision machinery and controls support industrial automation and semiconductor tool components; exhibiting is not a signed order. Organizer confirms October 26-31 at Tokyo Big Sight; exhibitor number was reported by CNA. Signed deals, qualification and equipment procurement are unknown. Location: Tokyo Big Sight, Tokyo, Japan (exhibition venue).</t>
+            <t xml:space="preserve">Foxconn and NVIDIA report 25% lower scheduling labor hours
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn and NVIDIA reported October 26 that scheduling labor hours fell 25% and molding engineering work fell 50% in selected manufacturing processes. A specified model-training task ran 2.48 times faster on DGX than an older H100 system; cross-factory validation was not disclosed. Applications span SMT, scheduling, automation, metrology and server AI training. NVIDIA cites an H100 comparison and one trillion tokens processed over 12 days; selected workflow outcomes are not factory-wide averages. Test sites, absolute baseline hours and line yield data remain undisclosed.</t>
           </r>
         </is>
       </c>
@@ -775,17 +775,54 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Metrology and process-power suppliers would verify baseline labor hours and site scope. Results cannot be generalized without controlled samples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="178" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">JIMTOF opens in Tokyo with 94 Taiwan exhibitors, association says
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">JIMTOF opened October 26 at Tokyo Big Sight, running through October 31. Taiwan's machine-tool association reported 94 participating companies covering CNC, metrology and automation; new orders were not disclosed. Precision machinery and controls support industrial automation and semiconductor tool components; exhibiting is not a signed order. Organizer confirms October 26-31 at Tokyo Big Sight; exhibitor number was reported by CNA. Signed deals, qualification and equipment procurement are unknown. Location: Tokyo Big Sight, Tokyo, Japan (exhibition venue).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C15" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Equipment-power and precision metrology suppliers would verify tool specifications and customer acceptance; participation does not prove sales.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="262" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+    <row r="16" ht="262" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -804,43 +841,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">NARLabs announced October 27 that its instrumentation center and Materials Analysis Technology Inc. (MSS) developed a coating approach to stabilize high-NA EUV metal-oxide-resist nanostructures for subsequent wafer cross-section analysis. NARLabs says it helped MSS enter major semiconductor suppliers' process chains, without customer acceptance, yield or deployment volumes. High-NA EUV metal-oxide-resist patterns require structural preservation during cross-section sample preparation, linking advanced lithography to metrology and microscopy. NARLabs describes stabilizing fragile patterned structures with coating prior to analysis. The disclosed research milestone is not evidence of a qualified high-volume manufacturing node. Comparative defect rates, tested resolution, fab qualification dates and commercial metrology orders were not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C15" s="6">
-        <v>46322</v>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Process-metrology, power and analysis-tool suppliers would examine material compatibility, specimen reproducibility and qualification. Research success does not establish volume tool contracts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="246" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Hongwei says specialized industrial lift orders now provide three years of visibility
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">On October 27, Hongwei Electric said its backlog for heavy-duty, cleanroom and automated material-handling lifts now offers three years of visibility, with orders on hand doubling versus 2025. It described semiconductor-related shipments as roughly 59% of the relevant mix, without disclosing absolute contract value or customer site details. Cleanroom, heavy-load and explosion-proof lifts support factory logistics and utilities, not front-end lithography or process equipment. Management said orders-to-shipments remained above one and reported sales to semiconductor and testing-related customers; three-year backlog visibility is a company estimate, not realized revenue. Absolute backlog units, contract values, delivery schedule and named project sites were not disclosed or independently verified.</t>
           </r>
         </is>
       </c>
@@ -849,7 +849,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industrial power and material-handling suppliers would seek delivery sites, load ratings and acceptance milestones. Backlog visibility is not recognized revenue or evidence of wafer-fab commissioning.</t>
+          <t xml:space="preserve">Process-metrology, power and analysis-tool suppliers would examine material compatibility, specimen reproducibility and qualification. Research success does not establish volume tool contracts.</t>
         </is>
       </c>
     </row>
@@ -868,6 +868,43 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Hongwei says specialized industrial lift orders now provide three years of visibility
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 27, Hongwei Electric said its backlog for heavy-duty, cleanroom and automated material-handling lifts now offers three years of visibility, with orders on hand doubling versus 2025. It described semiconductor-related shipments as roughly 59% of the relevant mix, without disclosing absolute contract value or customer site details. Cleanroom, heavy-load and explosion-proof lifts support factory logistics and utilities, not front-end lithography or process equipment. Management said orders-to-shipments remained above one and reported sales to semiconductor and testing-related customers; three-year backlog visibility is a company estimate, not realized revenue. Absolute backlog units, contract values, delivery schedule and named project sites were not disclosed or independently verified.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C17" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial power and material-handling suppliers would seek delivery sites, load ratings and acceptance milestones. Backlog visibility is not recognized revenue or evidence of wafer-fab commissioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="246" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Follow-up: CHPT reports nearly NT$400M Q3 advanced probe-card sales and 3x capacity target
 </t>
           </r>
@@ -878,43 +915,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">At an October 28 briefing, CHPT said advanced probe cards contributed nearly NT$400 million or 21% of Q3 revenue, while HPC products represented 65.9%. Capacity had doubled relative to end-2025 by August, with a threefold level targeted for Q1 2027, adding operational detail to the previous day's earnings. Probe cards, wafer test boards and high-power burn-in systems serve GPUs, TPUs, ASICs and CPO testing. Signal, power-integrity and temperature requirements differ by product. Management expects engineering CPU probe-card samples in November and targets volume production in 2027; CPO test interface talks involve more than five firms. These are stated qualification and commercial milestones, not completed acceptance. Absolute throughput, channel counts, accepted customers and high-power burn-in board volumes remain undisclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C17" s="6">
-        <v>46323</v>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Test-power, prober and burn-in suppliers would verify power density, channel requirements and qualification dates. A capacity multiple without absolute unit throughput cannot determine equipment volumes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="310" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Jin-An Machinery opens Longtan plant for ice-storage cooling and industrial unmanned systems
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">I-Mei affiliate Jin-An Machinery opened a new manufacturing building in Longtan, Taoyuan on October 28, following investment above NT$1 billion. The facility plans to make more than 20 off-peak ice-storage cooling systems for group factories; management claims a 25% to 30% reduction in peak electricity draw at an existing Longtan site, not a universal efficiency result. Ice-storage cooling shifts HVAC electricity loads from daytime to off-peak hours, rather than directly reducing chip-cooling load or total kWh. Unmanned systems and environmental tests are a separate line of work. The facility houses freeze-drying, thermal-storage and unmanned-system production. The above-NT$1B figure is a company-stated project total without tool/facility breakdown; 20-plus cooling systems are prospective production. Construction periods, individual system kW ratings, measured kWh and external customer acceptance counts are unavailable. Location: Longtan District, Taoyuan City, Taiwan, Jin-An manufacturing building (opened site, street address not verified).</t>
           </r>
         </is>
       </c>
@@ -923,17 +923,54 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Test-power, prober and burn-in suppliers would verify power density, channel requirements and qualification dates. A capacity multiple without absolute unit throughput cannot determine equipment volumes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="310" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Jin-An Machinery opens Longtan plant for ice-storage cooling and industrial unmanned systems
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">I-Mei affiliate Jin-An Machinery opened a new manufacturing building in Longtan, Taoyuan on October 28, following investment above NT$1 billion. The facility plans to make more than 20 off-peak ice-storage cooling systems for group factories; management claims a 25% to 30% reduction in peak electricity draw at an existing Longtan site, not a universal efficiency result. Ice-storage cooling shifts HVAC electricity loads from daytime to off-peak hours, rather than directly reducing chip-cooling load or total kWh. Unmanned systems and environmental tests are a separate line of work. The facility houses freeze-drying, thermal-storage and unmanned-system production. The above-NT$1B figure is a company-stated project total without tool/facility breakdown; 20-plus cooling systems are prospective production. Construction periods, individual system kW ratings, measured kWh and external customer acceptance counts are unavailable. Location: Longtan District, Taoyuan City, Taiwan, Jin-An manufacturing building (opened site, street address not verified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C19" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Industrial cooling, drives and power-controls suppliers would verify thermal-storage size, load profiles and peak demand calculations. A single site's reduction is not a universal data-center efficiency result.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="246" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
+    <row r="20" ht="246" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -955,22 +992,96 @@
           </r>
         </is>
       </c>
-      <c r="C19" s="6">
+      <c r="C20" s="6">
         <v>46324</v>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Industrial metrology, precision power and semiconductor-tool suppliers would distinguish applications and geography and verify deliveries. Book-to-bill indicates order flow, not the specific downstream deployment.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="400" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
+    <row r="21" ht="214" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">TSMC validates air-washer retrofits lowering pump power from 10 hp to 4 hp
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">In a report carried October 30, TSMC described air-washer retrofits reducing pump ratings from 10 to 4 horsepower, a 60% reduction for that pump. Operational validation was completed at Fab 6 and Advanced Backend Fab 7 by October; this is not a 60% reduction in total fab electricity use. Wafers; packaging/test; equipment; power; electricity; factories. A new wetted-media gravity-fed design reduces motorized pump load, according to TSMC, validated at Fab 6 and Advanced Backend Fab 7. The 60% saving is pump-specific rather than total wafer-fab energy use. Validated only in two named fabs with no total-site kWh baseline or complete rollout timeline.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C21" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facility-power and control suppliers would check modified pump load, controller specifications and maintenance constraints. Savings on a specific pump cannot be generalized to entire fabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="246" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan plans silicon-photonics test lab with overseas mutual validation in 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 30 Taiwan's National Development Council described a planned silicon-photonics validation laboratory targeting overseas inter-laboratory recognition in 2027 and OIF certification in 2028. Management cited existing offshore verification times of six months to two years; no new domestic lab has yet been commissioned. CPO; silicon photonics; testing; packaging; wafers; policy. Government officials cited overseas silicon-photonics validation taking six months to two years and proposed a domestic lab for CPO and optical interconnects. Mutual recognition and OIF certification remain future policy milestones. Lab address, capex, tool list, mutual-recognition terms and certification are pending. Location: Taipei, Taiwan; proposed silicon-photonics lab (specific site undisclosed).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C22" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Optical metrology and semiconductor-test firms would examine lab instrumentation, test standards and mutual-recognition rules. Future certification dates are not completed commercial qualification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="400" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -992,22 +1103,22 @@
           </r>
         </is>
       </c>
-      <c r="C20" s="6">
+      <c r="C23" s="6">
         <v>46317</v>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power, liquid-cooling and metrology suppliers would track the cable tender separately from Vietnam campus feasibility and site power agreements. Landing stations, anchor tenants, power contracts and construction permits are still missing.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="400" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
+    <row r="24" ht="400" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1029,22 +1140,22 @@
           </r>
         </is>
       </c>
-      <c r="C21" s="6">
+      <c r="C24" s="6">
         <v>46319</v>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power-conversion, UPS, power-quality and liquid-cooling suppliers would verify specific sites, permitted MW load, qualification and purchasing milestones. An aggregate intention without allocation cannot indicate equipment deliveries.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="214" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+    <row r="25" ht="214" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1066,22 +1177,22 @@
           </r>
         </is>
       </c>
-      <c r="C22" s="6">
+      <c r="C25" s="6">
         <v>46321</v>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power conversion and data-center suppliers need transmission specifications, storage designs and offtake terms. No finalized construction or financing plans are available.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="278" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">21</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
+    <row r="26" ht="278" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1103,22 +1214,22 @@
           </r>
         </is>
       </c>
-      <c r="C23" s="6">
+      <c r="C26" s="6">
         <v>46322</v>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Smart-factory power and test suppliers would check equipment type, whether transferred or newly built, and acceptance status. An intercompany book transaction cannot establish incremental production capacity.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="230" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
+    <row r="27" ht="230" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1140,22 +1251,22 @@
           </r>
         </is>
       </c>
-      <c r="C24" s="6">
+      <c r="C27" s="6">
         <v>46323</v>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Power and industrial metrology suppliers would separate group results from actual delivery of data-center modules and monitor later product qualification disclosures. Consolidated sales alone cannot quantify new rack deployment.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="262" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
+    <row r="28" ht="262" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1177,22 +1288,22 @@
           </r>
         </is>
       </c>
-      <c r="C25" s="6">
+      <c r="C28" s="6">
         <v>46323</v>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">UPS, power and liquid-cooling suppliers would verify the occupancy denominator, energized racks and power per cabinet. An 80% tenancy goal is not an equipment purchase count.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="262" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
+    <row r="29" ht="262" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">27</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1214,22 +1325,22 @@
           </r>
         </is>
       </c>
-      <c r="C26" s="6">
+      <c r="C29" s="6">
         <v>46324</v>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power and measurement suppliers would verify customers' grid readiness, electricians and equipment acceptance milestones. Inventory impairments reflect schedule and supply-mix issues, not necessarily product defects.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="262" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">25</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
+    <row r="30" ht="262" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1251,22 +1362,22 @@
           </r>
         </is>
       </c>
-      <c r="C27" s="6">
+      <c r="C30" s="6">
         <v>46324</v>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Server power, rack distribution and electronic test suppliers would verify actual procurement schedules and customer acceptance. Credit capacity cannot be translated into rack volumes or module purchase orders.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="326" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">26</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
+    <row r="31" ht="326" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1288,22 +1399,96 @@
           </r>
         </is>
       </c>
-      <c r="C28" s="6">
+      <c r="C31" s="6">
         <v>46324</v>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Rack-power, BBU and industrial-power suppliers would verify mechanical thermal, insulation, EMI and reliability qualifications. Production plans without order volumes do not establish deployed data-center power.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="342" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">27</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
+    <row r="32" ht="214" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Lite-On raises 2026 capex to NT$19.7B and discusses high-power supply production
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Lite-On on October 30 reported Q3 revenue of NT$57.4B and net profit of NT$7.4B, raising 2026 capex authorization to NT$19.7B. It said 8.5kW ASIC power supplies and BBUs are entering production; 800VDC Power Rack samples are planned for Q4 and its Vietnam plant targets a November opening. Power; BBU; servers; data centers; test; factories. The company said capex spent through September was about NT$13.1B, distinct from the NT$19.7B full-year budget. Vietnam's plant targets a November opening and the Texas site targets operations in Q2 2027. NT$19.7B is full-year budget, distinct from about NT$13.1B spent through September. Vietnam and U.S. site starts are future milestones.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C32" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-power conversion providers would check reliability and qualification milestones for 8.5kW modules, BBUs and 800VDC samples. Capex budgets do not establish completed deliveries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="210" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn says weekly AI-rack capacity doubled from 1,000 units
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At its October 30 Technology Day Foxconn said weekly AI-rack capacity doubled from roughly 1,000 units over a year, supported by differentiated assembly roles across Taiwan, Vietnam, the U.S. and Mexico. NVIDIA described more than ten factories involved in Vera Rubin manufacturing; actual shipments and qualified output remain undisclosed. ODM; servers; CPO; power; cooling; data centers. Foxconn described Level 1–12 production integration across Taiwan, Vietnam and North America. NVIDIA cited more than ten factories participating in Vera Rubin production without disclosing factory-level qualified output or customer deliveries. The doubling refers to reported weekly capacity rather than current shipments; Vera Rubin assembly plans remain in execution.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C33" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack-power, cooling and optical-test suppliers would verify Level 11/12 integration and CPO acceptance. Weekly nameplate capacity growth does not establish actual shipments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="342" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1325,22 +1510,22 @@
           </r>
         </is>
       </c>
-      <c r="C29" s="6">
+      <c r="C34" s="6">
         <v>46318</v>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Precision manufacturing metrology, optical packaging and data-center suppliers would need EBO ferrule yields, customer qualification and actual CPO production volumes. Placement funding and existing lens revenue do not reveal interconnect equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="374" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">28</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
+    <row r="35" ht="374" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1362,22 +1547,22 @@
           </r>
         </is>
       </c>
-      <c r="C30" s="6">
+      <c r="C35" s="6">
         <v>46320</v>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Server-rack and semiconductor-tool logistics and industrial power suppliers would distinguish urgent shipments from routine volumes and separate freight rates from fuel effects. Cargo revenue lacks an AI-specific mix and cannot establish production volume.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="230" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">29</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
+    <row r="36" ht="230" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1399,22 +1584,22 @@
           </r>
         </is>
       </c>
-      <c r="C31" s="6">
+      <c r="C36" s="6">
         <v>46321</v>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">SMT power, test and service suppliers would track any formal ownership and warranty changes. Reported bidding does not establish a contract transfer.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="262" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
+    <row r="37" ht="262" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1436,22 +1621,22 @@
           </r>
         </is>
       </c>
-      <c r="C32" s="6">
+      <c r="C37" s="6">
         <v>46322</v>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Packaging tool, test-power and metrology suppliers would check qualified package sizes, line requirements and actual delivery milestones. Q3 utilization and future expansion are separate measures, not equipment orders.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="230" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
+    <row r="38" ht="230" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1470,191 +1655,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">CHPT's board approved October 27 Q3 results showing NT$1.905 billion revenue, up 53.4% YoY, and NT$551 million attributable profit, up 100% YoY. Wafer probe cards accounted for 71% of Jan-Sep revenue and IC load boards for 21%; next-generation customer qualification data is not public. Wafer probe cards and IC load boards support wafer sorting and package test for memory and AI ASICs. Revenue mix is not production quantity. Its primary release reports 57.3% Q3 gross margin and roughly 35% operating margin, citing demand for customized AI testing interfaces. It gives growth rates without every absolute prior-year base. Next-generation probe-card customer roster, utilization, qualification times and new tool investments were not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C33" s="6">
-        <v>46322</v>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">High-frequency test-power and probe-card suppliers would seek channel-level signal/power-integrity specifications and qualification timelines. Sales mix cannot quantify tester procurement or throughput.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="246" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">WIN Semiconductors Q3 sales reach NT$5.859B; photodiode ramp ongoing
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">WIN Semiconductors announced October 28 Q3 revenue of NT$5.859 billion, gross margin 37.4% and attributable profit of NT$1.93 billion. Optical receiver photodiodes remain in early production ramp, with management pointing to larger-scale shipments in 2028; application-level volume was not reported. WIN's GaAs RF and receiver products serve satellite links, optical communications and data-center modules. Revenue growth is not evidence of new wafer-fab commissioning. Management said gross margin rose 9.2 percentage points from Q2 and profit increased around 98% sequentially. Q4 revenue guidance is low-single-digit sequential growth amid mixed handset demand. PD monthly shipments, yields, qualified customers and planned 2028 capacity allocations were not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C34" s="6">
-        <v>46323</v>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RF process-power and optical metrology suppliers would verify PD yields and receiver test bandwidth. Future volume projections cannot be inferred from consolidated profit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="326" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">33</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Follow-up: KYEC acquires Texas facility for US$79.35M and reports US$534M of tool purchases
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">On October 29, Taiwan's KYEC said its U.S. subsidiary AeternZ acquired a Texas site and building for US$79.35 million and disclosed about US$534 million in equipment and fab-utility purchases from Hon.Precision, EO Technics, KLA and TRANTEK. NVIDIA's previously announced US$1.1 billion capacity prepayment is background, while an April 2027 high-volume start remains a target. KYEC serves AI GPUs and ASICs through semiconductor testing, involving handlers, test-power systems, thermal management and facility utilities. A U.S. test site expands the geographic footprint of a Taiwan supplier, but the latest milestones are real-estate and equipment procurement. KYEC disclosed about 1,179,700 square feet of land and 489,494 square feet of buildings. Real-estate and tool transactions total roughly US$613 million as separate disclosed purchases; NVIDIA's US$1.1B prepayment is not an additional project cost to add to those figures. Exact Texas address, equipment acceptance dates, monthly test throughput, yields and first customer acceptance remain undisclosed. Location: AeternZ semiconductor test site in Texas, United States (land/building acquired; street address undisclosed).</t>
-          </r>
-        </is>
-      </c>
-      <c r="C35" s="6">
-        <v>46324</v>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Semiconductor test-power, precision metrology and thermal suppliers would verify purchased tool configuration, site bring-up and customer acceptance requirements. Procurement disclosures do not establish qualified 2027 output.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="342" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">34</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
-          </r>
-        </is>
-      </c>
-      <c r="C36" s="6">
-        <v>46319</v>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="294" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">35</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Reuters: Viettel fab lacks buildings and DUV equipment deal remains pending
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Reuters reported October 26 that no buildings have been constructed at Viettel's planned wafer fab outside Hanoi since a January groundbreaking and talks to purchase a DUV lithography tool from ASML remain unresolved. Sources doubt the 2027 trial-production target, whereas Viettel says progress remains in line with its plan. Vietnam already hosts Intel, Amkor and Hana Micron packaging/test sites. Viettel's proposed front-end fab would require lithography, deposition, etch, process power and utilities, distinct from installed packaging capacity. Reuters' site visit and satellite images found no buildings. Authorities previously estimated US$1.3 billion cost, a 2027 trial and full operation by 2030. Viettel says phased progress continues, while ASML has not confirmed a contract. DUV tool type, a signed procurement contract, construction permits, technology partner and validated trial date remain unknown. Location: Planned Viettel wafer fab site on the outskirts of Hanoi, Vietnam (industrial estate not specified).</t>
-          </r>
-        </is>
-      </c>
-      <c r="C37" s="6">
-        <v>46321</v>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wafer process-power and metrology suppliers would check signed equipment orders, process partnerships and building permits. Differing site evidence and developer statements leave the 2027 milestone unconfirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="246" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">36</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Faraday secures Samsung 2nm GAA design project, targets first revenue in H1 2027
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">On October 27, Faraday Technology announced a U.S. cloud AI chip non-recurring engineering project using Samsung's 2nm GAA foundry, with UMC and memory partners. Management described project value in the tens of millions of U.S. dollars and expects initial revenue recognition in H1 2027, without a precise contract value or qualified production date. The design project requires advanced-node IP and coordination across foundry and memory partners. UMC's participation does not make it the 2nm wafer foundry. Q3 revenue was NT$3.664B, gross margin 42.5% and attributable profit NT$279M. Management attributed margin changes partly to product mix and profit changes partly to non-operating valuation gains. Customer identity, package technology, exact NRE timing and chip shipment volumes were not given.</t>
           </r>
         </is>
       </c>
@@ -1663,11 +1663,11 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wafer process-power and advanced packaging test suppliers would verify actual foundry, package interface and qualification milestones. NRE contract value is not wafer manufacturing or equipment spending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="310" customHeight="1">
+          <t xml:space="preserve">High-frequency test-power and probe-card suppliers would seek channel-level signal/power-integrity specifications and qualification timelines. Sales mix cannot quantify tester procurement or throughput.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="246" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">37</t>
@@ -1682,16 +1682,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">UMC approves approximately US$3.2B additional capacity budget for Singapore and Tainan
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">On October 28, UMC's board approved around US$3.2 billion of additional expansion budget, intended to accelerate its Singapore and Tainan capacity plans, with no individual ramp dates. Q3 revenue was NT$74.24 billion, gross margin 34%, 12-inch-equivalent shipments over 1.2 million wafers and utilization 92%. The foundry serves mature and specialty nodes including 22/28nm technologies for power management, connectivity, silicon photonics and industrial controls. Board-authorized funding is not commissioned equipment or cash spent. UMC described US$2 billion 2026 capex separately from the new authorization. Guidance calls for Q4 shipment growth of 1% to 3% and utilization of 91% to 93%; 2027 blended ASP growth of 10% is a management expectation, not realized pricing. Site-by-site spending, tool awards, additional wafer starts, construction and commissioning dates are unknown; ASP and AI mix statements are forecasts. Location: Tainan Science Park, Taiwan, and Singapore facilities (regions for expansion; specific new building sites unspecified).</t>
+            <t xml:space="preserve">WIN Semiconductors Q3 sales reach NT$5.859B; photodiode ramp ongoing
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">WIN Semiconductors announced October 28 Q3 revenue of NT$5.859 billion, gross margin 37.4% and attributable profit of NT$1.93 billion. Optical receiver photodiodes remain in early production ramp, with management pointing to larger-scale shipments in 2028; application-level volume was not reported. WIN's GaAs RF and receiver products serve satellite links, optical communications and data-center modules. Revenue growth is not evidence of new wafer-fab commissioning. Management said gross margin rose 9.2 percentage points from Q2 and profit increased around 98% sequentially. Q4 revenue guidance is low-single-digit sequential growth amid mixed handset demand. PD monthly shipments, yields, qualified customers and planned 2028 capacity allocations were not disclosed.</t>
           </r>
         </is>
       </c>
@@ -1700,17 +1700,276 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">RF process-power and optical metrology suppliers would verify PD yields and receiver test bandwidth. Future volume projections cannot be inferred from consolidated profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="326" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Follow-up: KYEC acquires Texas facility for US$79.35M and reports US$534M of tool purchases
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 29, Taiwan's KYEC said its U.S. subsidiary AeternZ acquired a Texas site and building for US$79.35 million and disclosed about US$534 million in equipment and fab-utility purchases from Hon.Precision, EO Technics, KLA and TRANTEK. NVIDIA's previously announced US$1.1 billion capacity prepayment is background, while an April 2027 high-volume start remains a target. KYEC serves AI GPUs and ASICs through semiconductor testing, involving handlers, test-power systems, thermal management and facility utilities. A U.S. test site expands the geographic footprint of a Taiwan supplier, but the latest milestones are real-estate and equipment procurement. KYEC disclosed about 1,179,700 square feet of land and 489,494 square feet of buildings. Real-estate and tool transactions total roughly US$613 million as separate disclosed purchases; NVIDIA's US$1.1B prepayment is not an additional project cost to add to those figures. Exact Texas address, equipment acceptance dates, monthly test throughput, yields and first customer acceptance remain undisclosed. Location: AeternZ semiconductor test site in Texas, United States (land/building acquired; street address undisclosed).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C40" s="6">
+        <v>46324</v>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Semiconductor test-power, precision metrology and thermal suppliers would verify purchased tool configuration, site bring-up and customer acceptance requirements. Procurement disclosures do not establish qualified 2027 output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="178" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">MediaTek AI ASIC shipments and guidance
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 30 MediaTek said its first data-center ASIC began initial shipments in September and forecast US$2.5B of Q4 sales and US$16B in 2027. Q3 revenue was NT$168.058B with a 46.3% gross margin; a second ASIC targets Q1 2028 production. Chip design; foundry; packaging; data centers. Data-center accelerator designs depend on foundry, advanced packaging, substrates and interconnects. A second ASIC and customer were discussed without identifying the customer or wafer/package orders. Initial ASIC shipments have started, but future revenue, market share and a second chip ramp remain management forecasts.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C41" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-power and test-equipment suppliers would verify the foundry, package and customer qualification milestones. Future sales guidance does not quantify equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="194" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">ASE reports Q3 packaging/testing results and utilization
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">ASE Technology reported Q3 consolidated revenue around NT$244.2B on October 30 and described tight assembly, test and materials utilization in advanced applications. Packaging, testing and EMS segments must be distinguished, and actuals should not be conflated with guidance or analyst estimates. Packaging; testing; materials; servers. ASE consolidated revenue covers assembly, test, materials and electronics manufacturing services, not advanced packaging alone. Secondary reporting suggests constrained capacity without absolute tool/channel counts. The available source is a secondary report; original company disclosure is needed to verify segment results and utilization.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C42" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Packaging/test equipment and precision-power suppliers would seek utilization and customer acceptance by line. Available secondary reporting does not quantify additional advanced-packaging tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="342" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">41</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan envoy discusses Philippines semiconductor corridors and US$110B 2030 export target
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">At the TaiwanLink Fair in Makati on October 24, Taiwan's envoy discussed linking the Taiwan-Philippines and Luzon economic corridors for semiconductor cooperation. He cited the Philippines' goal of US$110 billion in annual electronics and semiconductor exports by 2030 and more than PHP45 billion of registered Taiwanese PEZA investment through end-2025; no new fab or assembly/test project approval was announced. The Philippines has electronics assembly, testing and industrial-park capacity, while Taiwan has chip design, wafer fabrication and equipment strengths. Economic-corridor linkages remain proposals in a speech, not finalized capex or facility approvals. The envoy cited historical PEZA registrations exceeding PHP45 billion and more than 20,000 direct jobs through December 2025, plus bilateral trade exceeding US$7 billion in the first eight months of 2026. These are dated reference figures, distinct from the October 24 cooperation remarks. No new Taiwan-Philippines semiconductor manufacturing contract, shared corridor construction plan, named manufacturer or committed project capital was disclosed. Location: Makati, Metro Manila, Philippines (TaiwanLink Fair opening event; specific venue unverified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C43" s="6">
+        <v>46319</v>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Packaging test-power and industrial controls suppliers would verify whether corridor discussions turn into permitted industrial projects, process specifications and qualified customers. Goals and historical PEZA investment do not quantify new equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="294" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">42</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Reuters: Viettel fab lacks buildings and DUV equipment deal remains pending
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Reuters reported October 26 that no buildings have been constructed at Viettel's planned wafer fab outside Hanoi since a January groundbreaking and talks to purchase a DUV lithography tool from ASML remain unresolved. Sources doubt the 2027 trial-production target, whereas Viettel says progress remains in line with its plan. Vietnam already hosts Intel, Amkor and Hana Micron packaging/test sites. Viettel's proposed front-end fab would require lithography, deposition, etch, process power and utilities, distinct from installed packaging capacity. Reuters' site visit and satellite images found no buildings. Authorities previously estimated US$1.3 billion cost, a 2027 trial and full operation by 2030. Viettel says phased progress continues, while ASML has not confirmed a contract. DUV tool type, a signed procurement contract, construction permits, technology partner and validated trial date remain unknown. Location: Planned Viettel wafer fab site on the outskirts of Hanoi, Vietnam (industrial estate not specified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C44" s="6">
+        <v>46321</v>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wafer process-power and metrology suppliers would check signed equipment orders, process partnerships and building permits. Differing site evidence and developer statements leave the 2027 milestone unconfirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="246" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Faraday secures Samsung 2nm GAA design project, targets first revenue in H1 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 27, Faraday Technology announced a U.S. cloud AI chip non-recurring engineering project using Samsung's 2nm GAA foundry, with UMC and memory partners. Management described project value in the tens of millions of U.S. dollars and expects initial revenue recognition in H1 2027, without a precise contract value or qualified production date. The design project requires advanced-node IP and coordination across foundry and memory partners. UMC's participation does not make it the 2nm wafer foundry. Q3 revenue was NT$3.664B, gross margin 42.5% and attributable profit NT$279M. Management attributed margin changes partly to product mix and profit changes partly to non-operating valuation gains. Customer identity, package technology, exact NRE timing and chip shipment volumes were not given.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C45" s="6">
+        <v>46322</v>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wafer process-power and advanced packaging test suppliers would verify actual foundry, package interface and qualification milestones. NRE contract value is not wafer manufacturing or equipment spending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="310" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">44</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">UMC approves approximately US$3.2B additional capacity budget for Singapore and Tainan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 28, UMC's board approved around US$3.2 billion of additional expansion budget, intended to accelerate its Singapore and Tainan capacity plans, with no individual ramp dates. Q3 revenue was NT$74.24 billion, gross margin 34%, 12-inch-equivalent shipments over 1.2 million wafers and utilization 92%. The foundry serves mature and specialty nodes including 22/28nm technologies for power management, connectivity, silicon photonics and industrial controls. Board-authorized funding is not commissioned equipment or cash spent. UMC described US$2 billion 2026 capex separately from the new authorization. Guidance calls for Q4 shipment growth of 1% to 3% and utilization of 91% to 93%; 2027 blended ASP growth of 10% is a management expectation, not realized pricing. Site-by-site spending, tool awards, additional wafer starts, construction and commissioning dates are unknown; ASP and AI mix statements are forecasts. Location: Tainan Science Park, Taiwan, and Singapore facilities (regions for expansion; specific new building sites unspecified).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C46" s="6">
+        <v>46323</v>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Process-power, metrology and packaging tool suppliers would verify equipment specifications and procurement schedules separately for Singapore and Tainan. Authorization and current utilization do not establish tool delivery.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="278" customHeight="1">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">38</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
+    <row r="47" ht="278" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">45</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1732,22 +1991,22 @@
           </r>
         </is>
       </c>
-      <c r="C40" s="6">
+      <c r="C47" s="6">
         <v>46310</v>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Server and test-equipment logistics providers would distinguish declarations, origin documentation and required permits. The investigation does not establish wrongdoing by any named manufacturer.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="342" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">39</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
+    <row r="48" ht="342" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">46</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1769,22 +2028,22 @@
           </r>
         </is>
       </c>
-      <c r="C41" s="6">
+      <c r="C48" s="6">
         <v>46324</v>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, test and fab-utility suppliers would verify closing, electrical capacity and qualification of any retrofitted cleanrooms. A real-estate purchase price does not identify tool orders.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="326" customHeight="1">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
+    <row r="49" ht="326" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">47</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1806,12 +2065,49 @@
           </r>
         </is>
       </c>
-      <c r="C42" s="6">
+      <c r="C49" s="6">
         <v>46324</v>
       </c>
-      <c r="D42" s="7" t="inlineStr">
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power and metrology businesses would examine subsector output, tool capex and electricity demand separately. An aggregate industry forecast does not quantify any individual equipment category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="226" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">King Slide authorizes NT$19.712B for Kaohsiung slide factories
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 30 King Slide said subsidiary Chuan Yi approved NT$19.712B in capex authorization for two Kaohsiung slide factories. A NT$11.733B construction amount awaits contractual pricing; NT$10.5B of equity financing and proposed convertible bonds are funding mechanisms, not additional construction cost. Components; servers; ODM; factories; investment. Subsidiary Chuan Yi approved third/fifth plant construction and equipment spending, with about NT$11.733B construction consideration pending negotiation and signing. NT$10.5B equity funding and proposed convertible bonds are financing instruments, not additional capex. Expansion is at budget and contracting stage; absolute output and acceptance dates were not announced. Location: Planned Chuan Yi factories 3 and 5 in Kaohsiung, Taiwan; specific addresses undisclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C50" s="6">
+        <v>46325</v>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manufacturing and metrology suppliers would verify slide output, automation specifications and tool acceptance. Board-approved capex does not establish production or executed equipment orders.</t>
         </is>
       </c>
     </row>

</xml_diff>